<commit_message>
fix: update vacuole and ER
</commit_message>
<xml_diff>
--- a/data/sce_compartment_curation/2026_curated/cytosol_annotations.xlsx
+++ b/data/sce_compartment_curation/2026_curated/cytosol_annotations.xlsx
@@ -441,7 +441,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>YGL180W</t>
+          <t>YPR017C</t>
         </is>
       </c>
     </row>
@@ -451,7 +451,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>YKL135C</t>
+          <t>YER162C</t>
         </is>
       </c>
     </row>
@@ -461,7 +461,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>YKL060C</t>
+          <t>YIL044C</t>
         </is>
       </c>
     </row>
@@ -471,7 +471,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>YNL163C</t>
+          <t>YHR030C</t>
         </is>
       </c>
     </row>
@@ -481,7 +481,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>YIR004W</t>
+          <t>YOR018W</t>
         </is>
       </c>
     </row>
@@ -491,7 +491,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>YDR300C</t>
+          <t>YBL041W</t>
         </is>
       </c>
     </row>
@@ -501,7 +501,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>YFR053C</t>
+          <t>YDR320C</t>
         </is>
       </c>
     </row>
@@ -511,7 +511,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>YBR214W</t>
+          <t>YHR150W</t>
         </is>
       </c>
     </row>
@@ -521,7 +521,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>YFL030W</t>
+          <t>YGR129W</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>YNR051C</t>
+          <t>YGL067W</t>
         </is>
       </c>
     </row>
@@ -541,7 +541,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>YGR074W</t>
+          <t>YGR048W</t>
         </is>
       </c>
     </row>
@@ -551,7 +551,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>YHR016C</t>
+          <t>YNL032W</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>YLR116W</t>
+          <t>YDR416W</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>YKR021W</t>
+          <t>YCR020C</t>
         </is>
       </c>
     </row>
@@ -581,7 +581,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>YFR021W</t>
+          <t>YDL226C</t>
         </is>
       </c>
     </row>
@@ -591,7 +591,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>YKL041W</t>
+          <t>YOL094C</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>YER020W</t>
+          <t>YGL066W</t>
         </is>
       </c>
     </row>
@@ -611,7 +611,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>YOR168W</t>
+          <t>YOL059W</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>YLL010C</t>
+          <t>YGR232W</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>YDR484W</t>
+          <t>YKR084C</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>YIL009C-A</t>
+          <t>YOR229W</t>
         </is>
       </c>
     </row>
@@ -651,7 +651,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>YDR195W</t>
+          <t>YCR027C</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>YIR012W</t>
+          <t>YDR363W-A</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>YPL262W</t>
+          <t>YBR019C</t>
         </is>
       </c>
     </row>
@@ -681,7 +681,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>YLL052C</t>
+          <t>YHR073W</t>
         </is>
       </c>
     </row>
@@ -691,7 +691,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>YGR248W</t>
+          <t>YMR079W</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>YDR044W</t>
+          <t>YLR044C</t>
         </is>
       </c>
     </row>
@@ -711,7 +711,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>YGL062W</t>
+          <t>YPL149W</t>
         </is>
       </c>
     </row>
@@ -721,7 +721,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>YGR037C</t>
+          <t>YFR008W</t>
         </is>
       </c>
     </row>
@@ -731,7 +731,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>YJL036W</t>
+          <t>YPL214C</t>
         </is>
       </c>
     </row>
@@ -741,7 +741,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>YDR189W</t>
+          <t>YLR376C</t>
         </is>
       </c>
     </row>
@@ -751,7 +751,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>YDR142C</t>
+          <t>YGR206W</t>
         </is>
       </c>
     </row>
@@ -761,7 +761,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>YNL273W</t>
+          <t>YNL163C</t>
         </is>
       </c>
     </row>
@@ -771,7 +771,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>YDR403W</t>
+          <t>YKL152C</t>
         </is>
       </c>
     </row>
@@ -781,7 +781,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>YOR115C</t>
+          <t>YMR037C</t>
         </is>
       </c>
     </row>
@@ -791,7 +791,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>YLR131C</t>
+          <t>YDR427W</t>
         </is>
       </c>
     </row>
@@ -801,7 +801,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>YLR153C</t>
+          <t>YGR234W</t>
         </is>
       </c>
     </row>
@@ -811,7 +811,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>YOL053W</t>
+          <t>YBR236C</t>
         </is>
       </c>
     </row>
@@ -821,7 +821,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>YJR141W</t>
+          <t>YDR388W</t>
         </is>
       </c>
     </row>
@@ -831,7 +831,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>YLL018C-A</t>
+          <t>YIR031C</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>YMR173W</t>
+          <t>YOR093C</t>
         </is>
       </c>
     </row>
@@ -851,7 +851,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>YNR016C</t>
+          <t>YHR085W</t>
         </is>
       </c>
     </row>
@@ -861,7 +861,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>YNL117W</t>
+          <t>YNL097C-B</t>
         </is>
       </c>
     </row>
@@ -871,7 +871,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>YER161C</t>
+          <t>YBR272C</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>YPR080W</t>
+          <t>YLR109W</t>
         </is>
       </c>
     </row>
@@ -891,7 +891,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>YNR010W</t>
+          <t>YMR159C</t>
         </is>
       </c>
     </row>
@@ -901,7 +901,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>YOR370C</t>
+          <t>YHR055C</t>
         </is>
       </c>
     </row>
@@ -911,7 +911,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>YDR517W</t>
+          <t>YKL113C</t>
         </is>
       </c>
     </row>
@@ -921,7 +921,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>YNL167C</t>
+          <t>YKL196C</t>
         </is>
       </c>
     </row>
@@ -931,7 +931,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>YPR010C-A</t>
+          <t>YOL062C</t>
         </is>
       </c>
     </row>
@@ -941,7 +941,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>YOL058W</t>
+          <t>YNL329C</t>
         </is>
       </c>
     </row>
@@ -951,7 +951,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>YHR109W</t>
+          <t>YDR517W</t>
         </is>
       </c>
     </row>
@@ -961,7 +961,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>YJL038C</t>
+          <t>YEL047C</t>
         </is>
       </c>
     </row>
@@ -971,7 +971,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>YLL038C</t>
+          <t>YJL168C</t>
         </is>
       </c>
     </row>
@@ -981,7 +981,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>YJL005W</t>
+          <t>YPR179C</t>
         </is>
       </c>
     </row>
@@ -991,7 +991,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>YDR244W</t>
+          <t>YGR059W</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>YHR170W</t>
+          <t>YKL135C</t>
         </is>
       </c>
     </row>
@@ -1011,7 +1011,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>YBR095C</t>
+          <t>YOR322C</t>
         </is>
       </c>
     </row>
@@ -1021,7 +1021,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>YIL007C</t>
+          <t>YNL051W</t>
         </is>
       </c>
     </row>
@@ -1031,7 +1031,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>YNL264C</t>
+          <t>YHR062C</t>
         </is>
       </c>
     </row>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>YDR464W</t>
+          <t>YOR119C</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>YDR427W</t>
+          <t>YGL169W</t>
         </is>
       </c>
     </row>
@@ -1061,7 +1061,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>YBR019C</t>
+          <t>YIL143C</t>
         </is>
       </c>
     </row>
@@ -1071,7 +1071,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>YBR149W</t>
+          <t>YPR185W</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1081,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>YPL153C</t>
+          <t>YEL048C</t>
         </is>
       </c>
     </row>
@@ -1091,7 +1091,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>YGR083C</t>
+          <t>YLL001W</t>
         </is>
       </c>
     </row>
@@ -1101,7 +1101,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>YIL044C</t>
+          <t>YNL231C</t>
         </is>
       </c>
     </row>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>YBR030W</t>
+          <t>YHR202W</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1121,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>YFR036W</t>
+          <t>YJL145W</t>
         </is>
       </c>
     </row>
@@ -1131,7 +1131,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>YGR198W</t>
+          <t>YGR192C</t>
         </is>
       </c>
     </row>
@@ -1141,7 +1141,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>YNL216W</t>
+          <t>YJL205C</t>
         </is>
       </c>
     </row>
@@ -1151,7 +1151,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>YPL096W</t>
+          <t>YCR033W</t>
         </is>
       </c>
     </row>
@@ -1161,7 +1161,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>YGR156W</t>
+          <t>YBR217W</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1171,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>YOR394W</t>
+          <t>YKR001C</t>
         </is>
       </c>
     </row>
@@ -1181,7 +1181,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>YHR160C</t>
+          <t>YBR080C</t>
         </is>
       </c>
     </row>
@@ -1191,7 +1191,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>YKR026C</t>
+          <t>YDR170C</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>YDR380W</t>
+          <t>YGR241C</t>
         </is>
       </c>
     </row>
@@ -1211,7 +1211,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>YNL051W</t>
+          <t>YGL013C</t>
         </is>
       </c>
     </row>
@@ -1221,7 +1221,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>YGL246C</t>
+          <t>YER046W</t>
         </is>
       </c>
     </row>
@@ -1231,7 +1231,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>YMR235C</t>
+          <t>YHL025W</t>
         </is>
       </c>
     </row>
@@ -1241,7 +1241,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>YGL211W</t>
+          <t>YJL006C</t>
         </is>
       </c>
     </row>
@@ -1251,7 +1251,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>YCL040W</t>
+          <t>YLR153C</t>
         </is>
       </c>
     </row>
@@ -1261,7 +1261,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>YDR069C</t>
+          <t>YBR067C</t>
         </is>
       </c>
     </row>
@@ -1271,7 +1271,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>YMR016C</t>
+          <t>YPL100W</t>
         </is>
       </c>
     </row>
@@ -1281,7 +1281,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>YAL035W</t>
+          <t>YDR069C</t>
         </is>
       </c>
     </row>
@@ -1291,7 +1291,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>YDR373W</t>
+          <t>YCR009C</t>
         </is>
       </c>
     </row>
@@ -1301,7 +1301,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>YOL059W</t>
+          <t>YPL153C</t>
         </is>
       </c>
     </row>
@@ -1311,7 +1311,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>YKL022C</t>
+          <t>YBR218C</t>
         </is>
       </c>
     </row>
@@ -1321,7 +1321,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>YMR037C</t>
+          <t>YOR113W</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1331,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>YDR255C</t>
+          <t>YLR011W</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1341,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>YER162C</t>
+          <t>YLR151C</t>
         </is>
       </c>
     </row>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>YGR057C</t>
+          <t>YMR165C</t>
         </is>
       </c>
     </row>
@@ -1361,7 +1361,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>YGR093W</t>
+          <t>YBR231C</t>
         </is>
       </c>
     </row>
@@ -1371,7 +1371,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>YNL240C</t>
+          <t>YFL013C</t>
         </is>
       </c>
     </row>
@@ -1381,7 +1381,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>YEL013W</t>
+          <t>YOR197W</t>
         </is>
       </c>
     </row>
@@ -1391,7 +1391,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>YIL026C</t>
+          <t>YER093C</t>
         </is>
       </c>
     </row>
@@ -1401,7 +1401,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>YPR017C</t>
+          <t>YPR144C</t>
         </is>
       </c>
     </row>
@@ -1411,7 +1411,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>YKR001C</t>
+          <t>YHR174W</t>
         </is>
       </c>
     </row>
@@ -1421,7 +1421,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>YIR007W</t>
+          <t>YGL047W</t>
         </is>
       </c>
     </row>
@@ -1431,7 +1431,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>YCR073W-A</t>
+          <t>YIR037W</t>
         </is>
       </c>
     </row>
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>YLR301W</t>
+          <t>YGL146C</t>
         </is>
       </c>
     </row>
@@ -1451,7 +1451,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>YDR487C</t>
+          <t>YCL002C</t>
         </is>
       </c>
     </row>
@@ -1461,7 +1461,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>YGL015C</t>
+          <t>YDR044W</t>
         </is>
       </c>
     </row>
@@ -1471,7 +1471,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>YLL001W</t>
+          <t>YNL035C</t>
         </is>
       </c>
     </row>
@@ -1481,7 +1481,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>YJL006C</t>
+          <t>YDR142C</t>
         </is>
       </c>
     </row>
@@ -1491,7 +1491,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>YKL197C</t>
+          <t>YLR438W</t>
         </is>
       </c>
     </row>
@@ -1501,7 +1501,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>YDR513W</t>
+          <t>YOR133W</t>
         </is>
       </c>
     </row>
@@ -1511,7 +1511,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>YBL041W</t>
+          <t>YDL009C</t>
         </is>
       </c>
     </row>
@@ -1521,7 +1521,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>YKL130C</t>
+          <t>YGL115W</t>
         </is>
       </c>
     </row>
@@ -1531,7 +1531,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>YNR070W</t>
+          <t>YNR031C</t>
         </is>
       </c>
     </row>
@@ -1541,7 +1541,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>YDL009C</t>
+          <t>YIR012W</t>
         </is>
       </c>
     </row>
@@ -1551,7 +1551,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>YMR038C</t>
+          <t>YER151C</t>
         </is>
       </c>
     </row>
@@ -1561,7 +1561,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>YCR033W</t>
+          <t>YLR310C</t>
         </is>
       </c>
     </row>
@@ -1571,7 +1571,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>YLR455W</t>
+          <t>YKL130C</t>
         </is>
       </c>
     </row>
@@ -1581,7 +1581,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>YGR068C</t>
+          <t>YBL058W</t>
         </is>
       </c>
     </row>
@@ -1591,7 +1591,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>YLL029W</t>
+          <t>YMR304W</t>
         </is>
       </c>
     </row>
@@ -1601,7 +1601,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>YKL067W</t>
+          <t>YLR240W</t>
         </is>
       </c>
     </row>
@@ -1611,7 +1611,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>YFL049W</t>
+          <t>YER161C</t>
         </is>
       </c>
     </row>
@@ -1621,7 +1621,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>YOR357C</t>
+          <t>YPL166W</t>
         </is>
       </c>
     </row>
@@ -1631,7 +1631,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>YGR274C</t>
+          <t>YPL204W</t>
         </is>
       </c>
     </row>
@@ -1641,7 +1641,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>YGR059W</t>
+          <t>YGL220W</t>
         </is>
       </c>
     </row>
@@ -1651,7 +1651,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>YMR029C</t>
+          <t>YBR056W</t>
         </is>
       </c>
     </row>
@@ -1661,7 +1661,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>YDR108W</t>
+          <t>YJL099W</t>
         </is>
       </c>
     </row>
@@ -1671,7 +1671,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>YPR180W</t>
+          <t>YBR030W</t>
         </is>
       </c>
     </row>
@@ -1681,7 +1681,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>YGL108C</t>
+          <t>YPL120W</t>
         </is>
       </c>
     </row>
@@ -1691,7 +1691,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>YBR105C</t>
+          <t>YLR043C</t>
         </is>
       </c>
     </row>
@@ -1701,7 +1701,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>YNL097C-B</t>
+          <t>YCL048W</t>
         </is>
       </c>
     </row>
@@ -1711,7 +1711,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>YER129W</t>
+          <t>YML097C</t>
         </is>
       </c>
     </row>
@@ -1721,7 +1721,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>YPR032W</t>
+          <t>YPR105C</t>
         </is>
       </c>
     </row>
@@ -1731,7 +1731,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>YGL124C</t>
+          <t>YDR189W</t>
         </is>
       </c>
     </row>
@@ -1741,7 +1741,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>YGR261C</t>
+          <t>YLR380W</t>
         </is>
       </c>
     </row>
@@ -1751,7 +1751,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>YJR104C</t>
+          <t>YIL131C</t>
         </is>
       </c>
     </row>
@@ -1761,7 +1761,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>YDR022C</t>
+          <t>YOR388C</t>
         </is>
       </c>
     </row>
@@ -1771,7 +1771,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>YHR055C</t>
+          <t>YOL058W</t>
         </is>
       </c>
     </row>
@@ -1781,7 +1781,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>YLR291C</t>
+          <t>YPL145C</t>
         </is>
       </c>
     </row>
@@ -1791,7 +1791,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>YIL084C</t>
+          <t>YGL195W</t>
         </is>
       </c>
     </row>
@@ -1801,7 +1801,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>YJL011C</t>
+          <t>YBL015W</t>
         </is>
       </c>
     </row>
@@ -1811,7 +1811,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>YDR073W</t>
+          <t>YJL011C</t>
         </is>
       </c>
     </row>
@@ -1821,7 +1821,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>YGL004C</t>
+          <t>YPL117C</t>
         </is>
       </c>
     </row>
@@ -1831,7 +1831,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>YKL206C</t>
+          <t>YGL005C</t>
         </is>
       </c>
     </row>
@@ -1841,7 +1841,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>YLL009C</t>
+          <t>YKL056C</t>
         </is>
       </c>
     </row>
@@ -1851,7 +1851,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>YCL058C</t>
+          <t>YLR039C</t>
         </is>
       </c>
     </row>
@@ -1861,7 +1861,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>YJL159W</t>
+          <t>YEL018W</t>
         </is>
       </c>
     </row>
@@ -1871,7 +1871,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>YPL065W</t>
+          <t>YMR061W</t>
         </is>
       </c>
     </row>
@@ -1881,7 +1881,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>YJL088W</t>
+          <t>YCL058C</t>
         </is>
       </c>
     </row>
@@ -1891,7 +1891,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>YCR043C</t>
+          <t>YBR214W</t>
         </is>
       </c>
     </row>
@@ -1901,7 +1901,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>YDR170C</t>
+          <t>YJL176C</t>
         </is>
       </c>
     </row>
@@ -1911,7 +1911,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>YHR085W</t>
+          <t>YBL001C</t>
         </is>
       </c>
     </row>
@@ -1921,7 +1921,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>YPR144C</t>
+          <t>YLR069C</t>
         </is>
       </c>
     </row>
@@ -1931,7 +1931,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>YBR164C</t>
+          <t>YBL018C</t>
         </is>
       </c>
     </row>
@@ -1941,7 +1941,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>YLR310C</t>
+          <t>YNL240C</t>
         </is>
       </c>
     </row>
@@ -1951,7 +1951,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>YPL061W</t>
+          <t>YOR323C</t>
         </is>
       </c>
     </row>
@@ -1961,7 +1961,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>YPL123C</t>
+          <t>YOR168W</t>
         </is>
       </c>
     </row>
@@ -1971,7 +1971,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>YOL062C</t>
+          <t>YFR036W</t>
         </is>
       </c>
     </row>
@@ -1981,7 +1981,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>YGL145W</t>
+          <t>YPL201C</t>
         </is>
       </c>
     </row>
@@ -2001,7 +2001,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>YER151C</t>
+          <t>YJL159W</t>
         </is>
       </c>
     </row>
@@ -2011,7 +2011,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>YOR113W</t>
+          <t>YGR198W</t>
         </is>
       </c>
     </row>
@@ -2021,7 +2021,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>YGR233C</t>
+          <t>YNL216W</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>YAL054C</t>
+          <t>YBL101C</t>
         </is>
       </c>
     </row>
@@ -2041,7 +2041,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>YGL146C</t>
+          <t>YLL009C</t>
         </is>
       </c>
     </row>
@@ -2051,7 +2051,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>YDL022W</t>
+          <t>YDL234C</t>
         </is>
       </c>
     </row>
@@ -2061,7 +2061,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>YDR174W</t>
+          <t>YOL138C</t>
         </is>
       </c>
     </row>
@@ -2071,7 +2071,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>YCL028W</t>
+          <t>YNL127W</t>
         </is>
       </c>
     </row>
@@ -2081,7 +2081,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>YNR035C</t>
+          <t>YHR019C</t>
         </is>
       </c>
     </row>
@@ -2091,7 +2091,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>YBL101C</t>
+          <t>YOR302W</t>
         </is>
       </c>
     </row>
@@ -2101,7 +2101,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>YDR372C</t>
+          <t>YGR068C</t>
         </is>
       </c>
     </row>
@@ -2111,7 +2111,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>YER040W</t>
+          <t>YNL290W</t>
         </is>
       </c>
     </row>
@@ -2121,7 +2121,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>YPL120W</t>
+          <t>YDR358W</t>
         </is>
       </c>
     </row>
@@ -2131,7 +2131,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>YIL131C</t>
+          <t>YGR239C</t>
         </is>
       </c>
     </row>
@@ -2141,7 +2141,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>YOR260W</t>
+          <t>YGR009C</t>
         </is>
       </c>
     </row>
@@ -2151,7 +2151,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>YNR031C</t>
+          <t>YHR160C</t>
         </is>
       </c>
     </row>
@@ -2161,7 +2161,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>YBL078C</t>
+          <t>YHR090C</t>
         </is>
       </c>
     </row>
@@ -2171,7 +2171,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>YMR159C</t>
+          <t>YJR104C</t>
         </is>
       </c>
     </row>
@@ -2181,7 +2181,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>YKR071C</t>
+          <t>YLL018C-A</t>
         </is>
       </c>
     </row>
@@ -2191,7 +2191,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>YER024W</t>
+          <t>YDL087C</t>
         </is>
       </c>
     </row>
@@ -2201,7 +2201,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>YML071C</t>
+          <t>YOR076C</t>
         </is>
       </c>
     </row>
@@ -2211,7 +2211,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>YDL022C-A</t>
+          <t>YGR019W</t>
         </is>
       </c>
     </row>
@@ -2221,7 +2221,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>YHR155W</t>
+          <t>YJL005W</t>
         </is>
       </c>
     </row>
@@ -2231,7 +2231,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>YKL069W</t>
+          <t>YKR021W</t>
         </is>
       </c>
     </row>
@@ -2241,7 +2241,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>YDL135C</t>
+          <t>YJR032W</t>
         </is>
       </c>
     </row>
@@ -2251,7 +2251,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>YMR208W</t>
+          <t>YBR151W</t>
         </is>
       </c>
     </row>
@@ -2261,7 +2261,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>YGL083W</t>
+          <t>YDR196C</t>
         </is>
       </c>
     </row>
@@ -2271,7 +2271,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>YIL041W</t>
+          <t>YGL258W</t>
         </is>
       </c>
     </row>
@@ -2281,7 +2281,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>YPL138C</t>
+          <t>YLR027C</t>
         </is>
       </c>
     </row>
@@ -2291,7 +2291,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>YBR172C</t>
+          <t>YKR026C</t>
         </is>
       </c>
     </row>
@@ -2301,7 +2301,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>YKL126W</t>
+          <t>YCL034W</t>
         </is>
       </c>
     </row>
@@ -2311,7 +2311,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>YPL051W</t>
+          <t>YDR380W</t>
         </is>
       </c>
     </row>
@@ -2321,7 +2321,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>YBL015W</t>
+          <t>YNR070W</t>
         </is>
       </c>
     </row>
@@ -2331,7 +2331,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>YNL127W</t>
+          <t>YHR133C</t>
         </is>
       </c>
     </row>
@@ -2341,7 +2341,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>YMR068W</t>
+          <t>YGR083C</t>
         </is>
       </c>
     </row>
@@ -2351,7 +2351,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>YGR009C</t>
+          <t>YGR274C</t>
         </is>
       </c>
     </row>
@@ -2361,7 +2361,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>YGR192C</t>
+          <t>YGR261C</t>
         </is>
       </c>
     </row>
@@ -2371,7 +2371,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>YER175C</t>
+          <t>YKL062W</t>
         </is>
       </c>
     </row>
@@ -2381,7 +2381,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>YOR323C</t>
+          <t>YJR006W</t>
         </is>
       </c>
     </row>
@@ -2391,7 +2391,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>YNL259C</t>
+          <t>YNL282W</t>
         </is>
       </c>
     </row>
@@ -2401,7 +2401,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>YDR334W</t>
+          <t>YBR149W</t>
         </is>
       </c>
     </row>
@@ -2411,7 +2411,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>YPL100W</t>
+          <t>YLL036C</t>
         </is>
       </c>
     </row>
@@ -2421,7 +2421,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>YDL192W</t>
+          <t>YER020W</t>
         </is>
       </c>
     </row>
@@ -2431,7 +2431,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>YNL227C</t>
+          <t>YHL043W</t>
         </is>
       </c>
     </row>
@@ -2441,7 +2441,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>YML113W</t>
+          <t>YNL207W</t>
         </is>
       </c>
     </row>
@@ -2451,7 +2451,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>YLR262C</t>
+          <t>YJR009C</t>
         </is>
       </c>
     </row>
@@ -2461,7 +2461,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>YGR270W</t>
+          <t>YFR022W</t>
         </is>
       </c>
     </row>
@@ -2471,7 +2471,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>YJL205C</t>
+          <t>YGL015C</t>
         </is>
       </c>
     </row>
@@ -2481,7 +2481,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>YNL183C</t>
+          <t>YDR180W</t>
         </is>
       </c>
     </row>
@@ -2491,7 +2491,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>YEL046C</t>
+          <t>YIL041W</t>
         </is>
       </c>
     </row>
@@ -2501,7 +2501,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>YHR206W</t>
+          <t>YDL022W</t>
         </is>
       </c>
     </row>
@@ -2511,7 +2511,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>YDR490C</t>
+          <t>YDR211W</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>YAR007C</t>
+          <t>YMR182C</t>
         </is>
       </c>
     </row>
@@ -2531,7 +2531,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>YMR079W</t>
+          <t>YMR208W</t>
         </is>
       </c>
     </row>
@@ -2541,7 +2541,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>YDR452W</t>
+          <t>YKL182W</t>
         </is>
       </c>
     </row>
@@ -2551,7 +2551,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>YJL102W</t>
+          <t>YLR330W</t>
         </is>
       </c>
     </row>
@@ -2561,7 +2561,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>YDL005C</t>
+          <t>YPR030W</t>
         </is>
       </c>
     </row>
@@ -2571,7 +2571,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>YIL143C</t>
+          <t>YIL026C</t>
         </is>
       </c>
     </row>
@@ -2581,7 +2581,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>YDR098C</t>
+          <t>YGL099W</t>
         </is>
       </c>
     </row>
@@ -2591,7 +2591,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>YDL100C</t>
+          <t>YNL293W</t>
         </is>
       </c>
     </row>
@@ -2601,7 +2601,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>YER057C</t>
+          <t>YNL247W</t>
         </is>
       </c>
     </row>
@@ -2611,7 +2611,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>YLR043C</t>
+          <t>YGL045W</t>
         </is>
       </c>
     </row>
@@ -2621,7 +2621,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>YMR182C</t>
+          <t>YHR155W</t>
         </is>
       </c>
     </row>
@@ -2631,7 +2631,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>YHR150W</t>
+          <t>YAL005C</t>
         </is>
       </c>
     </row>
@@ -2641,7 +2641,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>YOL094C</t>
+          <t>YGR248W</t>
         </is>
       </c>
     </row>
@@ -2651,7 +2651,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>YLR309C</t>
+          <t>YER040W</t>
         </is>
       </c>
     </row>
@@ -2661,7 +2661,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>YNL074C</t>
+          <t>YPL091W</t>
         </is>
       </c>
     </row>
@@ -2671,7 +2671,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>YHR073W</t>
+          <t>YLL024C</t>
         </is>
       </c>
     </row>
@@ -2681,7 +2681,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>YCR032W</t>
+          <t>YDR472W</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>YMR028W</t>
+          <t>YDR195W</t>
         </is>
       </c>
     </row>
@@ -2701,7 +2701,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>YPL204W</t>
+          <t>YDR295C</t>
         </is>
       </c>
     </row>
@@ -2711,7 +2711,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>YKR097W</t>
+          <t>YCL008C</t>
         </is>
       </c>
     </row>
@@ -2721,7 +2721,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>YHR133C</t>
+          <t>YNL117W</t>
         </is>
       </c>
     </row>
@@ -2731,7 +2731,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>YGR019W</t>
+          <t>YDR484W</t>
         </is>
       </c>
     </row>
@@ -2741,7 +2741,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>YOR322C</t>
+          <t>YML102W</t>
         </is>
       </c>
     </row>
@@ -2751,7 +2751,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>YPL070W</t>
+          <t>YLR131C</t>
         </is>
       </c>
     </row>
@@ -2761,7 +2761,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>YOR388C</t>
+          <t>YHR035W</t>
         </is>
       </c>
     </row>
@@ -2771,7 +2771,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>YGR234W</t>
+          <t>YDR141C</t>
         </is>
       </c>
     </row>
@@ -2781,7 +2781,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>YKL176C</t>
+          <t>YKL067W</t>
         </is>
       </c>
     </row>
@@ -2791,7 +2791,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>YDR353W</t>
+          <t>YNL167C</t>
         </is>
       </c>
     </row>
@@ -2801,7 +2801,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>YOR038C</t>
+          <t>YAR007C</t>
         </is>
       </c>
     </row>
@@ -2811,7 +2811,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>YGL258W</t>
+          <t>YGL008C</t>
         </is>
       </c>
     </row>
@@ -2821,7 +2821,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>YKL152C</t>
+          <t>YNL264C</t>
         </is>
       </c>
     </row>
@@ -2831,7 +2831,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>YMR070W</t>
+          <t>YNR010W</t>
         </is>
       </c>
     </row>
@@ -2841,7 +2841,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>YOR359W</t>
+          <t>YDR267C</t>
         </is>
       </c>
     </row>
@@ -2851,7 +2851,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>YDR180W</t>
+          <t>YGR037C</t>
         </is>
       </c>
     </row>
@@ -2861,7 +2861,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>YNL231C</t>
+          <t>YNL258C</t>
         </is>
       </c>
     </row>
@@ -2871,7 +2871,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>YBL001C</t>
+          <t>YPL138C</t>
         </is>
       </c>
     </row>
@@ -2881,7 +2881,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>YGL195W</t>
+          <t>YBL091C-A</t>
         </is>
       </c>
     </row>
@@ -2891,7 +2891,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>YBR231C</t>
+          <t>YDR073W</t>
         </is>
       </c>
     </row>
@@ -2901,7 +2901,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>YJL115W</t>
+          <t>YPL262W</t>
         </is>
       </c>
     </row>
@@ -2911,7 +2911,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>YDR096W</t>
+          <t>YER025W</t>
         </is>
       </c>
     </row>
@@ -2921,7 +2921,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>YPR030W</t>
+          <t>YOR094W</t>
         </is>
       </c>
     </row>
@@ -2931,7 +2931,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>YDR049W</t>
+          <t>YMR023C</t>
         </is>
       </c>
     </row>
@@ -2941,7 +2941,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>YGL045W</t>
+          <t>YMR120C</t>
         </is>
       </c>
     </row>
@@ -2951,7 +2951,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>YOR093C</t>
+          <t>YNL300W</t>
         </is>
       </c>
     </row>
@@ -2961,7 +2961,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>YBL058W</t>
+          <t>YKL059C</t>
         </is>
       </c>
     </row>
@@ -2971,7 +2971,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>YGR144W</t>
+          <t>YPR180W</t>
         </is>
       </c>
     </row>
@@ -2981,7 +2981,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>YLR151C</t>
+          <t>YJL088W</t>
         </is>
       </c>
     </row>
@@ -2991,7 +2991,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>YPL201C</t>
+          <t>YMR029C</t>
         </is>
       </c>
     </row>
@@ -3001,7 +3001,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>YLR069C</t>
+          <t>YLR262C</t>
         </is>
       </c>
     </row>
@@ -3011,7 +3011,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>YLL036C</t>
+          <t>YPR080W</t>
         </is>
       </c>
     </row>
@@ -3021,7 +3021,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>YNL242W</t>
+          <t>YHR016C</t>
         </is>
       </c>
     </row>
@@ -3031,7 +3031,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>YLR195C</t>
+          <t>YGR254W</t>
         </is>
       </c>
     </row>
@@ -3041,7 +3041,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>YOL081W</t>
+          <t>YNL227C</t>
         </is>
       </c>
     </row>
@@ -3051,7 +3051,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>YOL126C</t>
+          <t>YOR157C</t>
         </is>
       </c>
     </row>
@@ -3061,7 +3061,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>YGL220W</t>
+          <t>YCL055W</t>
         </is>
       </c>
     </row>
@@ -3071,7 +3071,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>YNL064C</t>
+          <t>YCL011C</t>
         </is>
       </c>
     </row>
@@ -3081,7 +3081,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>YNL258C</t>
+          <t>YDR218C</t>
         </is>
       </c>
     </row>
@@ -3091,7 +3091,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>YLR044C</t>
+          <t>YPL175W</t>
         </is>
       </c>
     </row>
@@ -3101,7 +3101,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>YGL099W</t>
+          <t>YDL022C-A</t>
         </is>
       </c>
     </row>
@@ -3111,7 +3111,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>YMR077C</t>
+          <t>YLR019W</t>
         </is>
       </c>
     </row>
@@ -3121,7 +3121,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>YHR030C</t>
+          <t>YGR142W</t>
         </is>
       </c>
     </row>
@@ -3131,7 +3131,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>YML102W</t>
+          <t>YGR252W</t>
         </is>
       </c>
     </row>
@@ -3141,7 +3141,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>YER023W</t>
+          <t>YKL126W</t>
         </is>
       </c>
     </row>
@@ -3151,7 +3151,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>YPL091W</t>
+          <t>YBL078C</t>
         </is>
       </c>
     </row>
@@ -3161,7 +3161,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>YKR084C</t>
+          <t>YEL022W</t>
         </is>
       </c>
     </row>
@@ -3171,7 +3171,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>YHR197W</t>
+          <t>YLL010C</t>
         </is>
       </c>
     </row>
@@ -3181,7 +3181,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>YOL138C</t>
+          <t>YGR209C</t>
         </is>
       </c>
     </row>
@@ -3191,7 +3191,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>YCL002C</t>
+          <t>YMR173W</t>
         </is>
       </c>
     </row>
@@ -3201,7 +3201,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>YBR152W</t>
+          <t>YIL063C</t>
         </is>
       </c>
     </row>
@@ -3211,7 +3211,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>YCL048W</t>
+          <t>YLR174W</t>
         </is>
       </c>
     </row>
@@ -3221,7 +3221,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>YBL075C</t>
+          <t>YDR490C</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>YJR072C</t>
+          <t>YPL070W</t>
         </is>
       </c>
     </row>
@@ -3241,7 +3241,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>YLR039C</t>
+          <t>YEL013W</t>
         </is>
       </c>
     </row>
@@ -3251,7 +3251,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>YGR232W</t>
+          <t>YDL135C</t>
         </is>
       </c>
     </row>
@@ -3261,7 +3261,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>YPR176C</t>
+          <t>YDL100C</t>
         </is>
       </c>
     </row>
@@ -3271,7 +3271,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>YPL084W</t>
+          <t>YKR020W</t>
         </is>
       </c>
     </row>
@@ -3281,7 +3281,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>YPR103W</t>
+          <t>YGR144W</t>
         </is>
       </c>
     </row>
@@ -3291,7 +3291,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>YDR141C</t>
+          <t>YPL123C</t>
         </is>
       </c>
     </row>
@@ -3301,7 +3301,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>YAL005C</t>
+          <t>YIL036W</t>
         </is>
       </c>
     </row>
@@ -3311,7 +3311,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>YEL021W</t>
+          <t>YJR072C</t>
         </is>
       </c>
     </row>
@@ -3321,7 +3321,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>YGL047W</t>
+          <t>YNL273W</t>
         </is>
       </c>
     </row>
@@ -3331,7 +3331,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>YBL076C</t>
+          <t>YDR513W</t>
         </is>
       </c>
     </row>
@@ -3341,7 +3341,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>YPL175W</t>
+          <t>YPR107C</t>
         </is>
       </c>
     </row>
@@ -3351,7 +3351,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>YHR171W</t>
+          <t>YBR289W</t>
         </is>
       </c>
     </row>
@@ -3361,7 +3361,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>YLR376C</t>
+          <t>YGL180W</t>
         </is>
       </c>
     </row>
@@ -3371,7 +3371,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>YDR392W</t>
+          <t>YKR080W</t>
         </is>
       </c>
     </row>
@@ -3381,7 +3381,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>YLR293C</t>
+          <t>YNL183C</t>
         </is>
       </c>
     </row>
@@ -3391,7 +3391,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>YHR019C</t>
+          <t>YGR134W</t>
         </is>
       </c>
     </row>
@@ -3401,7 +3401,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>YJL084C</t>
+          <t>YIR004W</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>YCL011C</t>
+          <t>YFR053C</t>
         </is>
       </c>
     </row>
@@ -3421,7 +3421,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>YKL196C</t>
+          <t>YML028W</t>
         </is>
       </c>
     </row>
@@ -3431,7 +3431,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>YBR217W</t>
+          <t>YPL051W</t>
         </is>
       </c>
     </row>
@@ -3441,7 +3441,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>YFR008W</t>
+          <t>YJL038C</t>
         </is>
       </c>
     </row>
@@ -3451,7 +3451,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>YDR311W</t>
+          <t>YFR021W</t>
         </is>
       </c>
     </row>
@@ -3461,7 +3461,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>YDL137W</t>
+          <t>YOL081W</t>
         </is>
       </c>
     </row>
@@ -3471,7 +3471,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>YLR260W</t>
+          <t>YDR096W</t>
         </is>
       </c>
     </row>
@@ -3481,7 +3481,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>YNL068C</t>
+          <t>YJL061W</t>
         </is>
       </c>
     </row>
@@ -3491,7 +3491,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>YPR105C</t>
+          <t>YJL121C</t>
         </is>
       </c>
     </row>
@@ -3501,7 +3501,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>YPR159C-A</t>
+          <t>YDR228C</t>
         </is>
       </c>
     </row>
@@ -3511,7 +3511,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>YPR179C</t>
+          <t>YBR261C</t>
         </is>
       </c>
     </row>
@@ -3521,7 +3521,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>YML097C</t>
+          <t>YDL005C</t>
         </is>
       </c>
     </row>
@@ -3531,7 +3531,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>YDR358W</t>
+          <t>YOL115W</t>
         </is>
       </c>
     </row>
@@ -3541,7 +3541,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>YLR011W</t>
+          <t>YLR309C</t>
         </is>
       </c>
     </row>
@@ -3551,7 +3551,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>YOR197W</t>
+          <t>YNR007C</t>
         </is>
       </c>
     </row>
@@ -3561,7 +3561,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>YFL068W</t>
+          <t>YGL211W</t>
         </is>
       </c>
     </row>
@@ -3571,7 +3571,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>YBR056W</t>
+          <t>YCR043C</t>
         </is>
       </c>
     </row>
@@ -3581,7 +3581,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>YDL065C</t>
+          <t>YOR274W</t>
         </is>
       </c>
     </row>
@@ -3591,7 +3591,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>YGL169W</t>
+          <t>YHR005C</t>
         </is>
       </c>
     </row>
@@ -3601,7 +3601,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>YJL061W</t>
+          <t>YDR216W</t>
         </is>
       </c>
     </row>
@@ -3611,7 +3611,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>YNR007C</t>
+          <t>YGR058W</t>
         </is>
       </c>
     </row>
@@ -3621,7 +3621,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>YFL014W</t>
+          <t>YGL124C</t>
         </is>
       </c>
     </row>
@@ -3631,7 +3631,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>YGL067W</t>
+          <t>YKL197C</t>
         </is>
       </c>
     </row>
@@ -3641,7 +3641,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>YLR330W</t>
+          <t>YOR359W</t>
         </is>
       </c>
     </row>
@@ -3651,7 +3651,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>YHR005C</t>
+          <t>YDR403W</t>
         </is>
       </c>
     </row>
@@ -3661,7 +3661,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>YDR218C</t>
+          <t>YGL253W</t>
         </is>
       </c>
     </row>
@@ -3671,7 +3671,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>YLR380W</t>
+          <t>YMR018W</t>
         </is>
       </c>
     </row>
@@ -3681,7 +3681,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>YDR363W-A</t>
+          <t>YPL088W</t>
         </is>
       </c>
     </row>
@@ -3691,7 +3691,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>YDR211W</t>
+          <t>YKL069W</t>
         </is>
       </c>
     </row>
@@ -3701,7 +3701,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>YMR043W</t>
+          <t>YKR097W</t>
         </is>
       </c>
     </row>
@@ -3711,7 +3711,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>YBR101C</t>
+          <t>YGR093W</t>
         </is>
       </c>
     </row>
@@ -3721,7 +3721,7 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>YNR049C</t>
+          <t>YBR164C</t>
         </is>
       </c>
     </row>
@@ -3731,7 +3731,7 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>YOR122C</t>
+          <t>YER057C</t>
         </is>
       </c>
     </row>
@@ -3741,7 +3741,7 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>YDR079C-A</t>
+          <t>YDR022C</t>
         </is>
       </c>
     </row>
@@ -3751,7 +3751,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>YLL024C</t>
+          <t>YCL028W</t>
         </is>
       </c>
     </row>
@@ -3761,7 +3761,7 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>YKR007W</t>
+          <t>YGL108C</t>
         </is>
       </c>
     </row>
@@ -3771,7 +3771,7 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>YHR090C</t>
+          <t>YGR057C</t>
         </is>
       </c>
     </row>
@@ -3781,7 +3781,7 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>YJR032W</t>
+          <t>YKR007W</t>
         </is>
       </c>
     </row>
@@ -3791,7 +3791,7 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>YHR018C</t>
+          <t>YOR370C</t>
         </is>
       </c>
     </row>
@@ -3801,7 +3801,7 @@
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>YBL018C</t>
+          <t>YPL061W</t>
         </is>
       </c>
     </row>
@@ -3811,7 +3811,7 @@
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>YNL290W</t>
+          <t>YDR372C</t>
         </is>
       </c>
     </row>
@@ -3821,7 +3821,7 @@
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>YNL247W</t>
+          <t>YLR377C</t>
         </is>
       </c>
     </row>
@@ -3831,7 +3831,7 @@
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>YER046W</t>
+          <t>YNL259C</t>
         </is>
       </c>
     </row>
@@ -3841,7 +3841,7 @@
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>YGR254W</t>
+          <t>YHR018C</t>
         </is>
       </c>
     </row>
@@ -3851,7 +3851,7 @@
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>YLR240W</t>
+          <t>YOR394W</t>
         </is>
       </c>
     </row>
@@ -3861,7 +3861,7 @@
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>YBL050W</t>
+          <t>YBR172C</t>
         </is>
       </c>
     </row>
@@ -3871,7 +3871,7 @@
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>YKL113C</t>
+          <t>YHR170W</t>
         </is>
       </c>
     </row>
@@ -3881,7 +3881,7 @@
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>YJL068C</t>
+          <t>YDL137W</t>
         </is>
       </c>
     </row>
@@ -3891,7 +3891,7 @@
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>YBR080C</t>
+          <t>YGR074W</t>
         </is>
       </c>
     </row>
@@ -3901,7 +3901,7 @@
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>YJL029C</t>
+          <t>YBL050W</t>
         </is>
       </c>
     </row>
@@ -3911,7 +3911,7 @@
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>YNL246W</t>
+          <t>YGR156W</t>
         </is>
       </c>
     </row>
@@ -3921,7 +3921,7 @@
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>YPL214C</t>
+          <t>YGR270W</t>
         </is>
       </c>
     </row>
@@ -3931,7 +3931,7 @@
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>YER007C-A</t>
+          <t>YIR007W</t>
         </is>
       </c>
     </row>
@@ -3941,7 +3941,7 @@
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>YMR018W</t>
+          <t>YER175C</t>
         </is>
       </c>
     </row>
@@ -3951,7 +3951,7 @@
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>YIR031C</t>
+          <t>YNR049C</t>
         </is>
       </c>
     </row>
@@ -3961,7 +3961,7 @@
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>YNL282W</t>
+          <t>YEL046C</t>
         </is>
       </c>
     </row>
@@ -3971,7 +3971,7 @@
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>YNL329C</t>
+          <t>YPL065W</t>
         </is>
       </c>
     </row>
@@ -3981,7 +3981,7 @@
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>YGR252W</t>
+          <t>YHR109W</t>
         </is>
       </c>
     </row>
@@ -3991,7 +3991,7 @@
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>YJR006W</t>
+          <t>YAL035W</t>
         </is>
       </c>
     </row>
@@ -4001,7 +4001,7 @@
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>YHR053C</t>
+          <t>YOR357C</t>
         </is>
       </c>
     </row>
@@ -4011,7 +4011,7 @@
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>YNR024W</t>
+          <t>YNR034W-A</t>
         </is>
       </c>
     </row>
@@ -4021,7 +4021,7 @@
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>YKR020W</t>
+          <t>YBR105C</t>
         </is>
       </c>
     </row>
@@ -4031,7 +4031,7 @@
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>YGR209C</t>
+          <t>YKR082W</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>YNL035C</t>
+          <t>YPL140C</t>
         </is>
       </c>
     </row>
@@ -4051,7 +4051,7 @@
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>YHR001W</t>
+          <t>YHR131C</t>
         </is>
       </c>
     </row>
@@ -4061,7 +4061,7 @@
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>YLR377C</t>
+          <t>YFL049W</t>
         </is>
       </c>
     </row>
@@ -4071,7 +4071,7 @@
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>YOR119C</t>
+          <t>YFL068W</t>
         </is>
       </c>
     </row>
@@ -4081,7 +4081,7 @@
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>YGR030C</t>
+          <t>YDR373W</t>
         </is>
       </c>
     </row>
@@ -4091,7 +4091,7 @@
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>YPL249C</t>
+          <t>YNL242W</t>
         </is>
       </c>
     </row>
@@ -4101,7 +4101,7 @@
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>YIR037W</t>
+          <t>YNL246W</t>
         </is>
       </c>
     </row>
@@ -4111,7 +4111,7 @@
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>YNL207W</t>
+          <t>YMR016C</t>
         </is>
       </c>
     </row>
@@ -4121,7 +4121,7 @@
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>YOL082W</t>
+          <t>YLR116W</t>
         </is>
       </c>
     </row>
@@ -4131,7 +4131,7 @@
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>YHR035W</t>
+          <t>YJL084C</t>
         </is>
       </c>
     </row>
@@ -4141,7 +4141,7 @@
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>YIL036W</t>
+          <t>YDL065C</t>
         </is>
       </c>
     </row>
@@ -4151,7 +4151,7 @@
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>YNL006W</t>
+          <t>YDR108W</t>
         </is>
       </c>
     </row>
@@ -4161,7 +4161,7 @@
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>YPL166W</t>
+          <t>YER129W</t>
         </is>
       </c>
     </row>
@@ -4171,7 +4171,7 @@
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>YEL018W</t>
+          <t>YOR115C</t>
         </is>
       </c>
     </row>
@@ -4181,7 +4181,7 @@
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>YHR062C</t>
+          <t>YJL031C</t>
         </is>
       </c>
     </row>
@@ -4191,7 +4191,7 @@
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>YGR241C</t>
+          <t>YLR028C</t>
         </is>
       </c>
     </row>
@@ -4201,7 +4201,7 @@
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>YDR177W</t>
+          <t>YGR233C</t>
         </is>
       </c>
     </row>
@@ -4211,7 +4211,7 @@
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>YIL104C</t>
+          <t>YKR071C</t>
         </is>
       </c>
     </row>
@@ -4221,7 +4221,7 @@
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t>YHR202W</t>
+          <t>YKL022C</t>
         </is>
       </c>
     </row>
@@ -4231,7 +4231,7 @@
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>YDR196C</t>
+          <t>YHR053C</t>
         </is>
       </c>
     </row>
@@ -4241,7 +4241,7 @@
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t>YBR236C</t>
+          <t>YJL052W</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t>YIL118W</t>
+          <t>YLR304C</t>
         </is>
       </c>
     </row>
@@ -4261,7 +4261,7 @@
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>YGL115W</t>
+          <t>YOR069W</t>
         </is>
       </c>
     </row>
@@ -4271,7 +4271,7 @@
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t>YOR069W</t>
+          <t>YKL176C</t>
         </is>
       </c>
     </row>
@@ -4281,7 +4281,7 @@
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t>YDR416W</t>
+          <t>YCL040W</t>
         </is>
       </c>
     </row>
@@ -4291,7 +4291,7 @@
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>YDL226C</t>
+          <t>YFL014W</t>
         </is>
       </c>
     </row>
@@ -4301,7 +4301,7 @@
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>YOR157C</t>
+          <t>YMR235C</t>
         </is>
       </c>
     </row>
@@ -4311,7 +4311,7 @@
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>YCL055W</t>
+          <t>YDL108W</t>
         </is>
       </c>
     </row>
@@ -4321,7 +4321,7 @@
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>YKL026C</t>
+          <t>YGL083W</t>
         </is>
       </c>
     </row>
@@ -4331,7 +4331,7 @@
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t>YEL022W</t>
+          <t>YGL095C</t>
         </is>
       </c>
     </row>
@@ -4341,7 +4341,7 @@
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t>YGR142W</t>
+          <t>YJL115W</t>
         </is>
       </c>
     </row>
@@ -4351,7 +4351,7 @@
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t>YJL031C</t>
+          <t>YOL126C</t>
         </is>
       </c>
     </row>
@@ -4361,7 +4361,7 @@
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t>YDR422C</t>
+          <t>YBR017C</t>
         </is>
       </c>
     </row>
@@ -4371,7 +4371,7 @@
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t>YIL063C</t>
+          <t>YLR301W</t>
         </is>
       </c>
     </row>
@@ -4381,7 +4381,7 @@
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t>YMR165C</t>
+          <t>YNL006W</t>
         </is>
       </c>
     </row>
@@ -4391,7 +4391,7 @@
       </c>
       <c r="B397" t="inlineStr">
         <is>
-          <t>YDL108W</t>
+          <t>YPR032W</t>
         </is>
       </c>
     </row>
@@ -4401,7 +4401,7 @@
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t>YKR082W</t>
+          <t>YDL126C</t>
         </is>
       </c>
     </row>
@@ -4411,7 +4411,7 @@
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t>YHL025W</t>
+          <t>YJL029C</t>
         </is>
       </c>
     </row>
@@ -4421,7 +4421,7 @@
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t>YPL088W</t>
+          <t>YGL062W</t>
         </is>
       </c>
     </row>
@@ -4431,7 +4431,7 @@
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t>YER093C</t>
+          <t>YIL009C-A</t>
         </is>
       </c>
     </row>
@@ -4441,7 +4441,7 @@
       </c>
       <c r="B402" t="inlineStr">
         <is>
-          <t>YCL018W</t>
+          <t>YFL045C</t>
         </is>
       </c>
     </row>
@@ -4451,7 +4451,7 @@
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t>YKR080W</t>
+          <t>YNR051C</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t>YMR076C</t>
+          <t>YDR244W</t>
         </is>
       </c>
     </row>
@@ -4471,7 +4471,7 @@
       </c>
       <c r="B405" t="inlineStr">
         <is>
-          <t>YGL112C</t>
+          <t>YLR293C</t>
         </is>
       </c>
     </row>
@@ -4481,7 +4481,7 @@
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t>YOR229W</t>
+          <t>YNL064C</t>
         </is>
       </c>
     </row>
@@ -4491,7 +4491,7 @@
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t>YKL059C</t>
+          <t>YMR038C</t>
         </is>
       </c>
     </row>
@@ -4501,7 +4501,7 @@
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>YLR109W</t>
+          <t>YDR177W</t>
         </is>
       </c>
     </row>
@@ -4511,7 +4511,7 @@
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>YDR172W</t>
+          <t>YCR073W-A</t>
         </is>
       </c>
     </row>
@@ -4521,7 +4521,7 @@
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>YMR061W</t>
+          <t>YMR068W</t>
         </is>
       </c>
     </row>
@@ -4531,7 +4531,7 @@
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>YER025W</t>
+          <t>YDR049W</t>
         </is>
       </c>
     </row>
@@ -4541,7 +4541,7 @@
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t>YOR302W</t>
+          <t>YIL084C</t>
         </is>
       </c>
     </row>
@@ -4551,7 +4551,7 @@
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>YCL008C</t>
+          <t>YER023W</t>
         </is>
       </c>
     </row>
@@ -4561,7 +4561,7 @@
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>YPL149W</t>
+          <t>YDR098C</t>
         </is>
       </c>
     </row>
@@ -4571,7 +4571,7 @@
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t>YDL126C</t>
+          <t>YKL075C</t>
         </is>
       </c>
     </row>
@@ -4581,7 +4581,7 @@
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t>YAR002W</t>
+          <t>YMR028W</t>
         </is>
       </c>
     </row>
@@ -4591,7 +4591,7 @@
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>YNL015W</t>
+          <t>YOR122C</t>
         </is>
       </c>
     </row>
@@ -4601,7 +4601,7 @@
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t>YNL293W</t>
+          <t>YOL083W</t>
         </is>
       </c>
     </row>
@@ -4611,7 +4611,7 @@
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>YHL043W</t>
+          <t>YDR487C</t>
         </is>
       </c>
     </row>
@@ -4621,7 +4621,7 @@
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t>YNL272C</t>
+          <t>YBL076C</t>
         </is>
       </c>
     </row>
@@ -4631,7 +4631,7 @@
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>YLR027C</t>
+          <t>YJL068C</t>
         </is>
       </c>
     </row>
@@ -4641,7 +4641,7 @@
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>YJR009C</t>
+          <t>YKL060C</t>
         </is>
       </c>
     </row>
@@ -4651,7 +4651,7 @@
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>YLR174W</t>
+          <t>YPR159C-A</t>
         </is>
       </c>
     </row>
@@ -4661,7 +4661,7 @@
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>YJL099W</t>
+          <t>YPL111W</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>YCR027C</t>
+          <t>YGL009C</t>
         </is>
       </c>
     </row>
@@ -4681,7 +4681,7 @@
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>YPL145C</t>
+          <t>YGL112C</t>
         </is>
       </c>
     </row>
@@ -4691,7 +4691,7 @@
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>YJL052W</t>
+          <t>YLL029W</t>
         </is>
       </c>
     </row>
@@ -4701,7 +4701,7 @@
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>YNL300W</t>
+          <t>YHR176W</t>
         </is>
       </c>
     </row>
@@ -4711,7 +4711,7 @@
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t>YKL062W</t>
+          <t>YGL004C</t>
         </is>
       </c>
     </row>
@@ -4721,7 +4721,7 @@
       </c>
       <c r="B430" t="inlineStr">
         <is>
-          <t>YFR004W</t>
+          <t>YNL272C</t>
         </is>
       </c>
     </row>
@@ -4731,7 +4731,7 @@
       </c>
       <c r="B431" t="inlineStr">
         <is>
-          <t>YNL032W</t>
+          <t>YDR300C</t>
         </is>
       </c>
     </row>
@@ -4741,7 +4741,7 @@
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t>YGR239C</t>
+          <t>YDR392W</t>
         </is>
       </c>
     </row>
@@ -4751,7 +4751,7 @@
       </c>
       <c r="B433" t="inlineStr">
         <is>
-          <t>YML131W</t>
+          <t>YML113W</t>
         </is>
       </c>
     </row>
@@ -4761,7 +4761,7 @@
       </c>
       <c r="B434" t="inlineStr">
         <is>
-          <t>YFL045C</t>
+          <t>YPL084W</t>
         </is>
       </c>
     </row>
@@ -4771,7 +4771,7 @@
       </c>
       <c r="B435" t="inlineStr">
         <is>
-          <t>YMR277W</t>
+          <t>YMR077C</t>
         </is>
       </c>
     </row>
@@ -4781,7 +4781,7 @@
       </c>
       <c r="B436" t="inlineStr">
         <is>
-          <t>YCR009C</t>
+          <t>YNL074C</t>
         </is>
       </c>
     </row>
@@ -4791,7 +4791,7 @@
       </c>
       <c r="B437" t="inlineStr">
         <is>
-          <t>YDL087C</t>
+          <t>YJL102W</t>
         </is>
       </c>
     </row>
@@ -4801,7 +4801,7 @@
       </c>
       <c r="B438" t="inlineStr">
         <is>
-          <t>YPL111W</t>
+          <t>YBR095C</t>
         </is>
       </c>
     </row>
@@ -4811,7 +4811,7 @@
       </c>
       <c r="B439" t="inlineStr">
         <is>
-          <t>YOR274W</t>
+          <t>YLR291C</t>
         </is>
       </c>
     </row>
@@ -4821,7 +4821,7 @@
       </c>
       <c r="B440" t="inlineStr">
         <is>
-          <t>YKL056C</t>
+          <t>YJL036W</t>
         </is>
       </c>
     </row>
@@ -4831,7 +4831,7 @@
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t>YOL083W</t>
+          <t>YPL096W</t>
         </is>
       </c>
     </row>
@@ -4841,7 +4841,7 @@
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t>YOR133W</t>
+          <t>YGR120C</t>
         </is>
       </c>
     </row>
@@ -4851,7 +4851,7 @@
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t>YBR131W</t>
+          <t>YDR079C-A</t>
         </is>
       </c>
     </row>
@@ -4861,7 +4861,7 @@
       </c>
       <c r="B444" t="inlineStr">
         <is>
-          <t>YJL044C</t>
+          <t>YNR035C</t>
         </is>
       </c>
     </row>
@@ -4871,7 +4871,7 @@
       </c>
       <c r="B445" t="inlineStr">
         <is>
-          <t>YLR028C</t>
+          <t>YPR103W</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="B446" t="inlineStr">
         <is>
-          <t>YGR134W</t>
+          <t>YIL104C</t>
         </is>
       </c>
     </row>
@@ -4891,7 +4891,7 @@
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t>YHR131C</t>
+          <t>YMR277W</t>
         </is>
       </c>
     </row>
@@ -4901,7 +4901,7 @@
       </c>
       <c r="B448" t="inlineStr">
         <is>
-          <t>YKR068C</t>
+          <t>YHR197W</t>
         </is>
       </c>
     </row>
@@ -4911,7 +4911,7 @@
       </c>
       <c r="B449" t="inlineStr">
         <is>
-          <t>YGR058W</t>
+          <t>YDR464W</t>
         </is>
       </c>
     </row>
@@ -4921,7 +4921,7 @@
       </c>
       <c r="B450" t="inlineStr">
         <is>
-          <t>YDR472W</t>
+          <t>YHR206W</t>
         </is>
       </c>
     </row>
@@ -4931,7 +4931,7 @@
       </c>
       <c r="B451" t="inlineStr">
         <is>
-          <t>YPL140C</t>
+          <t>YDR353W</t>
         </is>
       </c>
     </row>
@@ -4941,7 +4941,7 @@
       </c>
       <c r="B452" t="inlineStr">
         <is>
-          <t>YGR048W</t>
+          <t>YBL075C</t>
         </is>
       </c>
     </row>
@@ -4951,7 +4951,7 @@
       </c>
       <c r="B453" t="inlineStr">
         <is>
-          <t>YDR267C</t>
+          <t>YGL246C</t>
         </is>
       </c>
     </row>
@@ -4961,7 +4961,7 @@
       </c>
       <c r="B454" t="inlineStr">
         <is>
-          <t>YFL013C</t>
+          <t>YLR396C</t>
         </is>
       </c>
     </row>
@@ -4971,7 +4971,7 @@
       </c>
       <c r="B455" t="inlineStr">
         <is>
-          <t>YKL182W</t>
+          <t>YFL030W</t>
         </is>
       </c>
     </row>
@@ -4981,7 +4981,7 @@
       </c>
       <c r="B456" t="inlineStr">
         <is>
-          <t>YER048C</t>
+          <t>YLL052C</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4991,7 @@
       </c>
       <c r="B457" t="inlineStr">
         <is>
-          <t>YDL234C</t>
+          <t>YAL054C</t>
         </is>
       </c>
     </row>
@@ -5001,7 +5001,7 @@
       </c>
       <c r="B458" t="inlineStr">
         <is>
-          <t>YGR129W</t>
+          <t>YNR016C</t>
         </is>
       </c>
     </row>
@@ -5011,7 +5011,7 @@
       </c>
       <c r="B459" t="inlineStr">
         <is>
-          <t>YOL115W</t>
+          <t>YHR171W</t>
         </is>
       </c>
     </row>
@@ -5021,7 +5021,7 @@
       </c>
       <c r="B460" t="inlineStr">
         <is>
-          <t>YGL013C</t>
+          <t>YDR452W</t>
         </is>
       </c>
     </row>
@@ -5031,7 +5031,7 @@
       </c>
       <c r="B461" t="inlineStr">
         <is>
-          <t>YOL055C</t>
+          <t>YMR043W</t>
         </is>
       </c>
     </row>
@@ -5041,7 +5041,7 @@
       </c>
       <c r="B462" t="inlineStr">
         <is>
-          <t>YPR185W</t>
+          <t>YBR131W</t>
         </is>
       </c>
     </row>
@@ -5051,7 +5051,7 @@
       </c>
       <c r="B463" t="inlineStr">
         <is>
-          <t>YBR272C</t>
+          <t>YHR001W</t>
         </is>
       </c>
     </row>
@@ -5061,7 +5061,7 @@
       </c>
       <c r="B464" t="inlineStr">
         <is>
-          <t>YJL176C</t>
+          <t>YCL018W</t>
         </is>
       </c>
     </row>
@@ -5071,7 +5071,7 @@
       </c>
       <c r="B465" t="inlineStr">
         <is>
-          <t>YBR218C</t>
+          <t>YER007C-A</t>
         </is>
       </c>
     </row>
@@ -5081,7 +5081,7 @@
       </c>
       <c r="B466" t="inlineStr">
         <is>
-          <t>YJL121C</t>
+          <t>YJR102C</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="B467" t="inlineStr">
         <is>
-          <t>YBR017C</t>
+          <t>YOR260W</t>
         </is>
       </c>
     </row>
@@ -5101,7 +5101,7 @@
       </c>
       <c r="B468" t="inlineStr">
         <is>
-          <t>YDR320C</t>
+          <t>YKL041W</t>
         </is>
       </c>
     </row>
@@ -5111,7 +5111,7 @@
       </c>
       <c r="B469" t="inlineStr">
         <is>
-          <t>YDL106C</t>
+          <t>YJL208C</t>
         </is>
       </c>
     </row>
@@ -5121,7 +5121,7 @@
       </c>
       <c r="B470" t="inlineStr">
         <is>
-          <t>YPR107C</t>
+          <t>YPL203W</t>
         </is>
       </c>
     </row>
@@ -5131,7 +5131,7 @@
       </c>
       <c r="B471" t="inlineStr">
         <is>
-          <t>YLR396C</t>
+          <t>YBR152W</t>
         </is>
       </c>
     </row>
@@ -5141,7 +5141,7 @@
       </c>
       <c r="B472" t="inlineStr">
         <is>
-          <t>YBL091C-A</t>
+          <t>YDR334W</t>
         </is>
       </c>
     </row>
@@ -5151,7 +5151,7 @@
       </c>
       <c r="B473" t="inlineStr">
         <is>
-          <t>YBR067C</t>
+          <t>YLL038C</t>
         </is>
       </c>
     </row>
@@ -5161,7 +5161,7 @@
       </c>
       <c r="B474" t="inlineStr">
         <is>
-          <t>YGL253W</t>
+          <t>YNR023W</t>
         </is>
       </c>
     </row>
@@ -5171,7 +5171,7 @@
       </c>
       <c r="B475" t="inlineStr">
         <is>
-          <t>YNR034W-A</t>
+          <t>YKR068C</t>
         </is>
       </c>
     </row>
@@ -5181,7 +5181,7 @@
       </c>
       <c r="B476" t="inlineStr">
         <is>
-          <t>YDR228C</t>
+          <t>YPL249C</t>
         </is>
       </c>
     </row>
@@ -5191,7 +5191,7 @@
       </c>
       <c r="B477" t="inlineStr">
         <is>
-          <t>YOR018W</t>
+          <t>YDR422C</t>
         </is>
       </c>
     </row>
@@ -5201,7 +5201,7 @@
       </c>
       <c r="B478" t="inlineStr">
         <is>
-          <t>YCR020C</t>
+          <t>YDL192W</t>
         </is>
       </c>
     </row>
@@ -5211,7 +5211,7 @@
       </c>
       <c r="B479" t="inlineStr">
         <is>
-          <t>YEL048C</t>
+          <t>YJR141W</t>
         </is>
       </c>
     </row>
@@ -5221,7 +5221,7 @@
       </c>
       <c r="B480" t="inlineStr">
         <is>
-          <t>YML028W</t>
+          <t>YPR010C-A</t>
         </is>
       </c>
     </row>
@@ -5231,7 +5231,7 @@
       </c>
       <c r="B481" t="inlineStr">
         <is>
-          <t>YNR023W</t>
+          <t>YGR030C</t>
         </is>
       </c>
     </row>
@@ -5241,7 +5241,7 @@
       </c>
       <c r="B482" t="inlineStr">
         <is>
-          <t>YDR165W</t>
+          <t>YPL231W</t>
         </is>
       </c>
     </row>
@@ -5251,7 +5251,7 @@
       </c>
       <c r="B483" t="inlineStr">
         <is>
-          <t>YOR094W</t>
+          <t>YDL106C</t>
         </is>
       </c>
     </row>
@@ -5261,7 +5261,7 @@
       </c>
       <c r="B484" t="inlineStr">
         <is>
-          <t>YDR216W</t>
+          <t>YDR172W</t>
         </is>
       </c>
     </row>
@@ -5271,7 +5271,7 @@
       </c>
       <c r="B485" t="inlineStr">
         <is>
-          <t>YPL203W</t>
+          <t>YIL007C</t>
         </is>
       </c>
     </row>
@@ -5281,7 +5281,7 @@
       </c>
       <c r="B486" t="inlineStr">
         <is>
-          <t>YFR022W</t>
+          <t>YMR070W</t>
         </is>
       </c>
     </row>
@@ -5291,7 +5291,7 @@
       </c>
       <c r="B487" t="inlineStr">
         <is>
-          <t>YMR120C</t>
+          <t>YCR032W</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="B488" t="inlineStr">
         <is>
-          <t>YPL117C</t>
+          <t>YNR024W</t>
         </is>
       </c>
     </row>
@@ -5311,7 +5311,7 @@
       </c>
       <c r="B489" t="inlineStr">
         <is>
-          <t>YMR304W</t>
+          <t>YDR311W</t>
         </is>
       </c>
     </row>
@@ -5321,7 +5321,7 @@
       </c>
       <c r="B490" t="inlineStr">
         <is>
-          <t>YOR076C</t>
+          <t>YKL206C</t>
         </is>
       </c>
     </row>
@@ -5331,7 +5331,7 @@
       </c>
       <c r="B491" t="inlineStr">
         <is>
-          <t>YBR289W</t>
+          <t>YLR455W</t>
         </is>
       </c>
     </row>
@@ -5341,7 +5341,7 @@
       </c>
       <c r="B492" t="inlineStr">
         <is>
-          <t>YHR176W</t>
+          <t>YOL055C</t>
         </is>
       </c>
     </row>
@@ -5351,7 +5351,7 @@
       </c>
       <c r="B493" t="inlineStr">
         <is>
-          <t>YGL008C</t>
+          <t>YAR002W</t>
         </is>
       </c>
     </row>
@@ -5361,7 +5361,7 @@
       </c>
       <c r="B494" t="inlineStr">
         <is>
-          <t>YCL034W</t>
+          <t>YMR076C</t>
         </is>
       </c>
     </row>
@@ -5371,7 +5371,7 @@
       </c>
       <c r="B495" t="inlineStr">
         <is>
-          <t>YGL095C</t>
+          <t>YLR260W</t>
         </is>
       </c>
     </row>
@@ -5381,7 +5381,7 @@
       </c>
       <c r="B496" t="inlineStr">
         <is>
-          <t>YJL168C</t>
+          <t>YPR176C</t>
         </is>
       </c>
     </row>
@@ -5391,7 +5391,7 @@
       </c>
       <c r="B497" t="inlineStr">
         <is>
-          <t>YDR388W</t>
+          <t>YDR255C</t>
         </is>
       </c>
     </row>
@@ -5401,7 +5401,7 @@
       </c>
       <c r="B498" t="inlineStr">
         <is>
-          <t>YBR151W</t>
+          <t>YBR101C</t>
         </is>
       </c>
     </row>
@@ -5411,7 +5411,7 @@
       </c>
       <c r="B499" t="inlineStr">
         <is>
-          <t>YLR438W</t>
+          <t>YOL053W</t>
         </is>
       </c>
     </row>
@@ -5421,7 +5421,7 @@
       </c>
       <c r="B500" t="inlineStr">
         <is>
-          <t>YJL145W</t>
+          <t>YER024W</t>
         </is>
       </c>
     </row>
@@ -5431,7 +5431,7 @@
       </c>
       <c r="B501" t="inlineStr">
         <is>
-          <t>YGL066W</t>
+          <t>YLR195C</t>
         </is>
       </c>
     </row>
@@ -5441,7 +5441,7 @@
       </c>
       <c r="B502" t="inlineStr">
         <is>
-          <t>YDR295C</t>
+          <t>YIL118W</t>
         </is>
       </c>
     </row>
@@ -5451,7 +5451,7 @@
       </c>
       <c r="B503" t="inlineStr">
         <is>
-          <t>YJL208C</t>
+          <t>YGL145W</t>
         </is>
       </c>
     </row>
@@ -5461,7 +5461,7 @@
       </c>
       <c r="B504" t="inlineStr">
         <is>
-          <t>YJR102C</t>
+          <t>YER048C</t>
         </is>
       </c>
     </row>
@@ -5471,7 +5471,7 @@
       </c>
       <c r="B505" t="inlineStr">
         <is>
-          <t>YPL231W</t>
+          <t>YML131W</t>
         </is>
       </c>
     </row>
@@ -5481,7 +5481,7 @@
       </c>
       <c r="B506" t="inlineStr">
         <is>
-          <t>YMR023C</t>
+          <t>YKL026C</t>
         </is>
       </c>
     </row>
@@ -5491,7 +5491,7 @@
       </c>
       <c r="B507" t="inlineStr">
         <is>
-          <t>YGL005C</t>
+          <t>YNL068C</t>
         </is>
       </c>
     </row>
@@ -5501,7 +5501,7 @@
       </c>
       <c r="B508" t="inlineStr">
         <is>
-          <t>YGR206W</t>
+          <t>YJL044C</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="B509" t="inlineStr">
         <is>
-          <t>YKL075C</t>
+          <t>YDR165W</t>
         </is>
       </c>
     </row>
@@ -5521,7 +5521,7 @@
       </c>
       <c r="B510" t="inlineStr">
         <is>
-          <t>YGR120C</t>
+          <t>YOL082W</t>
         </is>
       </c>
     </row>
@@ -5531,7 +5531,7 @@
       </c>
       <c r="B511" t="inlineStr">
         <is>
-          <t>YLR304C</t>
+          <t>YEL021W</t>
         </is>
       </c>
     </row>
@@ -5541,7 +5541,7 @@
       </c>
       <c r="B512" t="inlineStr">
         <is>
-          <t>YGL009C</t>
+          <t>YDR174W</t>
         </is>
       </c>
     </row>
@@ -5551,7 +5551,7 @@
       </c>
       <c r="B513" t="inlineStr">
         <is>
-          <t>YEL047C</t>
+          <t>YNL015W</t>
         </is>
       </c>
     </row>
@@ -5561,7 +5561,7 @@
       </c>
       <c r="B514" t="inlineStr">
         <is>
-          <t>YHR174W</t>
+          <t>YOR038C</t>
         </is>
       </c>
     </row>
@@ -5571,7 +5571,7 @@
       </c>
       <c r="B515" t="inlineStr">
         <is>
-          <t>YLR019W</t>
+          <t>YML071C</t>
         </is>
       </c>
     </row>
@@ -5581,7 +5581,7 @@
       </c>
       <c r="B516" t="inlineStr">
         <is>
-          <t>YBR261C</t>
+          <t>YFR004W</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: update vocuole not ER
</commit_message>
<xml_diff>
--- a/data/sce_compartment_curation/2026_curated/cytosol_annotations.xlsx
+++ b/data/sce_compartment_curation/2026_curated/cytosol_annotations.xlsx
@@ -441,7 +441,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>YPR017C</t>
+          <t>YNR070W</t>
         </is>
       </c>
     </row>
@@ -451,7 +451,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>YER162C</t>
+          <t>YBR131W</t>
         </is>
       </c>
     </row>
@@ -461,7 +461,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>YIL044C</t>
+          <t>YLR260W</t>
         </is>
       </c>
     </row>
@@ -471,7 +471,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>YHR030C</t>
+          <t>YBL091C-A</t>
         </is>
       </c>
     </row>
@@ -481,7 +481,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>YOR018W</t>
+          <t>YOR323C</t>
         </is>
       </c>
     </row>
@@ -491,7 +491,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>YBL041W</t>
+          <t>YPR010C-A</t>
         </is>
       </c>
     </row>
@@ -501,7 +501,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>YDR320C</t>
+          <t>YDL192W</t>
         </is>
       </c>
     </row>
@@ -511,7 +511,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>YHR150W</t>
+          <t>YGL004C</t>
         </is>
       </c>
     </row>
@@ -521,7 +521,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>YGR129W</t>
+          <t>YGR019W</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>YGL067W</t>
+          <t>YDR141C</t>
         </is>
       </c>
     </row>
@@ -541,7 +541,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>YGR048W</t>
+          <t>YML102W</t>
         </is>
       </c>
     </row>
@@ -551,7 +551,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>YNL032W</t>
+          <t>YPL231W</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>YDR416W</t>
+          <t>YMR070W</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>YCR020C</t>
+          <t>YDR044W</t>
         </is>
       </c>
     </row>
@@ -581,7 +581,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>YDL226C</t>
+          <t>YCL048W</t>
         </is>
       </c>
     </row>
@@ -591,7 +591,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>YOL094C</t>
+          <t>YJL006C</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>YGL066W</t>
+          <t>YER046W</t>
         </is>
       </c>
     </row>
@@ -611,7 +611,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>YOL059W</t>
+          <t>YKL206C</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>YGR232W</t>
+          <t>YLL052C</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>YKR084C</t>
+          <t>YGR120C</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>YOR229W</t>
+          <t>YCR032W</t>
         </is>
       </c>
     </row>
@@ -651,7 +651,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>YCR027C</t>
+          <t>YLR019W</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>YDR363W-A</t>
+          <t>YPL149W</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>YBR019C</t>
+          <t>YFR004W</t>
         </is>
       </c>
     </row>
@@ -681,7 +681,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>YHR073W</t>
+          <t>YHR131C</t>
         </is>
       </c>
     </row>
@@ -691,7 +691,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>YMR079W</t>
+          <t>YLR291C</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>YLR044C</t>
+          <t>YNR031C</t>
         </is>
       </c>
     </row>
@@ -711,7 +711,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>YPL149W</t>
+          <t>YGR192C</t>
         </is>
       </c>
     </row>
@@ -721,7 +721,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>YFR008W</t>
+          <t>YGR252W</t>
         </is>
       </c>
     </row>
@@ -731,7 +731,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>YPL214C</t>
+          <t>YGR232W</t>
         </is>
       </c>
     </row>
@@ -741,7 +741,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>YLR376C</t>
+          <t>YJL208C</t>
         </is>
       </c>
     </row>
@@ -751,7 +751,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>YGR206W</t>
+          <t>YLL018C-A</t>
         </is>
       </c>
     </row>
@@ -761,7 +761,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>YNL163C</t>
+          <t>YNR034W-A</t>
         </is>
       </c>
     </row>
@@ -771,7 +771,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>YKL152C</t>
+          <t>YMR173W</t>
         </is>
       </c>
     </row>
@@ -781,7 +781,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>YMR037C</t>
+          <t>YPR017C</t>
         </is>
       </c>
     </row>
@@ -791,7 +791,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>YDR427W</t>
+          <t>YDR267C</t>
         </is>
       </c>
     </row>
@@ -801,7 +801,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>YGR234W</t>
+          <t>YHR085W</t>
         </is>
       </c>
     </row>
@@ -811,7 +811,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>YBR236C</t>
+          <t>YJL099W</t>
         </is>
       </c>
     </row>
@@ -821,7 +821,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>YDR388W</t>
+          <t>YOR018W</t>
         </is>
       </c>
     </row>
@@ -831,7 +831,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>YIR031C</t>
+          <t>YGR274C</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>YOR093C</t>
+          <t>YER175C</t>
         </is>
       </c>
     </row>
@@ -851,7 +851,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>YHR085W</t>
+          <t>YDR358W</t>
         </is>
       </c>
     </row>
@@ -861,7 +861,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>YNL097C-B</t>
+          <t>YKL126W</t>
         </is>
       </c>
     </row>
@@ -871,7 +871,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>YBR272C</t>
+          <t>YDR300C</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>YLR109W</t>
+          <t>YCR009C</t>
         </is>
       </c>
     </row>
@@ -891,7 +891,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>YMR159C</t>
+          <t>YIL063C</t>
         </is>
       </c>
     </row>
@@ -901,7 +901,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>YHR055C</t>
+          <t>YGR254W</t>
         </is>
       </c>
     </row>
@@ -911,7 +911,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>YKL113C</t>
+          <t>YHR005C</t>
         </is>
       </c>
     </row>
@@ -921,7 +921,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>YKL196C</t>
+          <t>YDR216W</t>
         </is>
       </c>
     </row>
@@ -931,7 +931,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>YOL062C</t>
+          <t>YER162C</t>
         </is>
       </c>
     </row>
@@ -941,7 +941,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>YNL329C</t>
+          <t>YDR388W</t>
         </is>
       </c>
     </row>
@@ -951,7 +951,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>YDR517W</t>
+          <t>YGL009C</t>
         </is>
       </c>
     </row>
@@ -961,7 +961,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>YEL047C</t>
+          <t>YGL180W</t>
         </is>
       </c>
     </row>
@@ -971,7 +971,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>YJL168C</t>
+          <t>YKR021W</t>
         </is>
       </c>
     </row>
@@ -981,7 +981,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>YPR179C</t>
+          <t>YEL048C</t>
         </is>
       </c>
     </row>
@@ -991,7 +991,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>YGR059W</t>
+          <t>YLR043C</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>YKL135C</t>
+          <t>YDR211W</t>
         </is>
       </c>
     </row>
@@ -1011,7 +1011,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>YOR322C</t>
+          <t>YGL146C</t>
         </is>
       </c>
     </row>
@@ -1021,7 +1021,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>YNL051W</t>
+          <t>YMR182C</t>
         </is>
       </c>
     </row>
@@ -1031,7 +1031,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>YHR062C</t>
+          <t>YDR170C</t>
         </is>
       </c>
     </row>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>YOR119C</t>
+          <t>YDL137W</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>YGL169W</t>
+          <t>YER048C</t>
         </is>
       </c>
     </row>
@@ -1061,7 +1061,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>YIL143C</t>
+          <t>YBR101C</t>
         </is>
       </c>
     </row>
@@ -1071,7 +1071,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>YPR185W</t>
+          <t>YPL214C</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1081,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>YEL048C</t>
+          <t>YDL100C</t>
         </is>
       </c>
     </row>
@@ -1091,7 +1091,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>YLL001W</t>
+          <t>YGL169W</t>
         </is>
       </c>
     </row>
@@ -1101,7 +1101,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>YNL231C</t>
+          <t>YHR019C</t>
         </is>
       </c>
     </row>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>YHR202W</t>
+          <t>YGL005C</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1121,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>YJL145W</t>
+          <t>YER025W</t>
         </is>
       </c>
     </row>
@@ -1131,7 +1131,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>YGR192C</t>
+          <t>YJR006W</t>
         </is>
       </c>
     </row>
@@ -1141,7 +1141,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>YJL205C</t>
+          <t>YKL059C</t>
         </is>
       </c>
     </row>
@@ -1151,7 +1151,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>YCR033W</t>
+          <t>YMR079W</t>
         </is>
       </c>
     </row>
@@ -1161,7 +1161,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>YBR217W</t>
+          <t>YGR233C</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1171,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>YKR001C</t>
+          <t>YHR155W</t>
         </is>
       </c>
     </row>
@@ -1181,7 +1181,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>YBR080C</t>
+          <t>YBR019C</t>
         </is>
       </c>
     </row>
@@ -1191,7 +1191,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>YDR170C</t>
+          <t>YNR007C</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>YGR241C</t>
+          <t>YFL068W</t>
         </is>
       </c>
     </row>
@@ -1211,7 +1211,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>YGL013C</t>
+          <t>YOL126C</t>
         </is>
       </c>
     </row>
@@ -1221,7 +1221,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>YER046W</t>
+          <t>YKR001C</t>
         </is>
       </c>
     </row>
@@ -1231,7 +1231,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>YHL025W</t>
+          <t>YFR053C</t>
         </is>
       </c>
     </row>
@@ -1241,7 +1241,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>YJL006C</t>
+          <t>YML113W</t>
         </is>
       </c>
     </row>
@@ -1251,7 +1251,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>YLR153C</t>
+          <t>YFR036W</t>
         </is>
       </c>
     </row>
@@ -1261,7 +1261,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>YBR067C</t>
+          <t>YDL135C</t>
         </is>
       </c>
     </row>
@@ -1271,7 +1271,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>YPL100W</t>
+          <t>YKR020W</t>
         </is>
       </c>
     </row>
@@ -1281,7 +1281,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>YDR069C</t>
+          <t>YPR179C</t>
         </is>
       </c>
     </row>
@@ -1291,7 +1291,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>YCR009C</t>
+          <t>YDR096W</t>
         </is>
       </c>
     </row>
@@ -1301,7 +1301,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>YPL153C</t>
+          <t>YKL096W-A</t>
         </is>
       </c>
     </row>
@@ -1311,7 +1311,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>YBR218C</t>
+          <t>YPL145C</t>
         </is>
       </c>
     </row>
@@ -1321,7 +1321,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>YOR113W</t>
+          <t>YHR090C</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1331,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>YLR011W</t>
+          <t>YDR049W</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1341,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>YLR151C</t>
+          <t>YDR334W</t>
         </is>
       </c>
     </row>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>YMR165C</t>
+          <t>YML097C</t>
         </is>
       </c>
     </row>
@@ -1361,7 +1361,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>YBR231C</t>
+          <t>YOR157C</t>
         </is>
       </c>
     </row>
@@ -1371,7 +1371,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>YFL013C</t>
+          <t>YNL032W</t>
         </is>
       </c>
     </row>
@@ -1381,7 +1381,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>YOR197W</t>
+          <t>YFR022W</t>
         </is>
       </c>
     </row>
@@ -1391,7 +1391,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>YER093C</t>
+          <t>YJR009C</t>
         </is>
       </c>
     </row>
@@ -1401,7 +1401,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>YPR144C</t>
+          <t>YFR008W</t>
         </is>
       </c>
     </row>
@@ -1411,7 +1411,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>YHR174W</t>
+          <t>YNL272C</t>
         </is>
       </c>
     </row>
@@ -1421,7 +1421,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>YGL047W</t>
+          <t>YBL076C</t>
         </is>
       </c>
     </row>
@@ -1431,7 +1431,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>YIR037W</t>
+          <t>YGR083C</t>
         </is>
       </c>
     </row>
@@ -1441,7 +1441,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>YGL146C</t>
+          <t>YMR077C</t>
         </is>
       </c>
     </row>
@@ -1451,7 +1451,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>YCL002C</t>
+          <t>YPL204W</t>
         </is>
       </c>
     </row>
@@ -1461,7 +1461,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>YDR044W</t>
+          <t>YOL081W</t>
         </is>
       </c>
     </row>
@@ -1471,7 +1471,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>YNL035C</t>
+          <t>YNL117W</t>
         </is>
       </c>
     </row>
@@ -1481,7 +1481,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>YDR142C</t>
+          <t>YJR104C</t>
         </is>
       </c>
     </row>
@@ -1491,7 +1491,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>YLR438W</t>
+          <t>YGL211W</t>
         </is>
       </c>
     </row>
@@ -1501,7 +1501,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>YOR133W</t>
+          <t>YMR165C</t>
         </is>
       </c>
     </row>
@@ -1511,7 +1511,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>YDL009C</t>
+          <t>YPR032W</t>
         </is>
       </c>
     </row>
@@ -1521,7 +1521,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>YGL115W</t>
+          <t>YJL084C</t>
         </is>
       </c>
     </row>
@@ -1531,7 +1531,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>YNR031C</t>
+          <t>YBL050W</t>
         </is>
       </c>
     </row>
@@ -1541,7 +1541,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>YIR012W</t>
+          <t>YPR107C</t>
         </is>
       </c>
     </row>
@@ -1551,7 +1551,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>YER151C</t>
+          <t>YGR206W</t>
         </is>
       </c>
     </row>
@@ -1561,7 +1561,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>YLR310C</t>
+          <t>YDR177W</t>
         </is>
       </c>
     </row>
@@ -1571,7 +1571,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>YKL130C</t>
+          <t>YLL038C</t>
         </is>
       </c>
     </row>
@@ -1581,7 +1581,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>YBL058W</t>
+          <t>YNL064C</t>
         </is>
       </c>
     </row>
@@ -1591,7 +1591,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>YMR304W</t>
+          <t>YDR108W</t>
         </is>
       </c>
     </row>
@@ -1601,7 +1601,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>YLR240W</t>
+          <t>YBL015W</t>
         </is>
       </c>
     </row>
@@ -1611,7 +1611,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>YER161C</t>
+          <t>YGL195W</t>
         </is>
       </c>
     </row>
@@ -1621,7 +1621,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>YPL166W</t>
+          <t>YNL163C</t>
         </is>
       </c>
     </row>
@@ -1631,7 +1631,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>YPL204W</t>
+          <t>YGR239C</t>
         </is>
       </c>
     </row>
@@ -1641,7 +1641,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>YGL220W</t>
+          <t>YPL166W</t>
         </is>
       </c>
     </row>
@@ -1651,7 +1651,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>YBR056W</t>
+          <t>YHR174W</t>
         </is>
       </c>
     </row>
@@ -1661,7 +1661,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>YJL099W</t>
+          <t>YJL168C</t>
         </is>
       </c>
     </row>
@@ -1671,7 +1671,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>YBR030W</t>
+          <t>YDL022W</t>
         </is>
       </c>
     </row>
@@ -1681,7 +1681,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>YPL120W</t>
+          <t>YKL197C</t>
         </is>
       </c>
     </row>
@@ -1691,7 +1691,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>YLR043C</t>
+          <t>YHR171W</t>
         </is>
       </c>
     </row>
@@ -1701,7 +1701,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>YCL048W</t>
+          <t>YPL140C</t>
         </is>
       </c>
     </row>
@@ -1711,7 +1711,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>YML097C</t>
+          <t>YMR038C</t>
         </is>
       </c>
     </row>
@@ -1721,7 +1721,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>YPR105C</t>
+          <t>YDR353W</t>
         </is>
       </c>
     </row>
@@ -1731,7 +1731,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>YDR189W</t>
+          <t>YNR049C</t>
         </is>
       </c>
     </row>
@@ -1741,7 +1741,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>YLR380W</t>
+          <t>YLR011W</t>
         </is>
       </c>
     </row>
@@ -1751,7 +1751,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>YIL131C</t>
+          <t>YGR030C</t>
         </is>
       </c>
     </row>
@@ -1761,7 +1761,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>YOR388C</t>
+          <t>YIL131C</t>
         </is>
       </c>
     </row>
@@ -1771,7 +1771,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>YOL058W</t>
+          <t>YGL067W</t>
         </is>
       </c>
     </row>
@@ -1781,7 +1781,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>YPL145C</t>
+          <t>YLR380W</t>
         </is>
       </c>
     </row>
@@ -1791,7 +1791,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>YGL195W</t>
+          <t>YJL115W</t>
         </is>
       </c>
     </row>
@@ -1801,7 +1801,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>YBL015W</t>
+          <t>YDL126C</t>
         </is>
       </c>
     </row>
@@ -1811,7 +1811,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>YJL011C</t>
+          <t>YLR293C</t>
         </is>
       </c>
     </row>
@@ -1821,7 +1821,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>YPL117C</t>
+          <t>YKL152C</t>
         </is>
       </c>
     </row>
@@ -1831,7 +1831,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>YGL005C</t>
+          <t>YHR176W</t>
         </is>
       </c>
     </row>
@@ -1841,7 +1841,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>YKL056C</t>
+          <t>YGL108C</t>
         </is>
       </c>
     </row>
@@ -1851,7 +1851,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>YLR039C</t>
+          <t>YJR072C</t>
         </is>
       </c>
     </row>
@@ -1861,7 +1861,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>YEL018W</t>
+          <t>YBL075C</t>
         </is>
       </c>
     </row>
@@ -1871,7 +1871,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>YMR061W</t>
+          <t>YGR142W</t>
         </is>
       </c>
     </row>
@@ -1881,7 +1881,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>YCL058C</t>
+          <t>YGL083W</t>
         </is>
       </c>
     </row>
@@ -1891,7 +1891,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>YBR214W</t>
+          <t>YGR248W</t>
         </is>
       </c>
     </row>
@@ -1901,7 +1901,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>YJL176C</t>
+          <t>YHL025W</t>
         </is>
       </c>
     </row>
@@ -1911,7 +1911,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>YBL001C</t>
+          <t>YJL068C</t>
         </is>
       </c>
     </row>
@@ -1921,7 +1921,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>YLR069C</t>
+          <t>YLR174W</t>
         </is>
       </c>
     </row>
@@ -1931,7 +1931,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>YBL018C</t>
+          <t>YDR363W-A</t>
         </is>
       </c>
     </row>
@@ -1941,7 +1941,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>YNL240C</t>
+          <t>YGL062W</t>
         </is>
       </c>
     </row>
@@ -1951,7 +1951,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>YOR323C</t>
+          <t>YOL058W</t>
         </is>
       </c>
     </row>
@@ -1961,7 +1961,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>YOR168W</t>
+          <t>YOR197W</t>
         </is>
       </c>
     </row>
@@ -1971,7 +1971,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>YFR036W</t>
+          <t>YER161C</t>
         </is>
       </c>
     </row>
@@ -1981,7 +1981,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>YPL201C</t>
+          <t>YLR069C</t>
         </is>
       </c>
     </row>
@@ -1991,7 +1991,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>YKL096W-A</t>
+          <t>YKR080W</t>
         </is>
       </c>
     </row>
@@ -2001,7 +2001,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>YJL159W</t>
+          <t>YGL008C</t>
         </is>
       </c>
     </row>
@@ -2011,7 +2011,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>YGR198W</t>
+          <t>YCR027C</t>
         </is>
       </c>
     </row>
@@ -2021,7 +2021,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>YNL216W</t>
+          <t>YHR062C</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>YBL101C</t>
+          <t>YMR159C</t>
         </is>
       </c>
     </row>
@@ -2041,7 +2041,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>YLL009C</t>
+          <t>YEL022W</t>
         </is>
       </c>
     </row>
@@ -2051,7 +2051,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>YDL234C</t>
+          <t>YHR109W</t>
         </is>
       </c>
     </row>
@@ -2061,7 +2061,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>YOL138C</t>
+          <t>YJR102C</t>
         </is>
       </c>
     </row>
@@ -2071,7 +2071,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>YNL127W</t>
+          <t>YJR032W</t>
         </is>
       </c>
     </row>
@@ -2081,7 +2081,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>YHR019C</t>
+          <t>YPL175W</t>
         </is>
       </c>
     </row>
@@ -2091,7 +2091,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>YOR302W</t>
+          <t>YBR217W</t>
         </is>
       </c>
     </row>
@@ -2101,7 +2101,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>YGR068C</t>
+          <t>YCL008C</t>
         </is>
       </c>
     </row>
@@ -2111,7 +2111,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>YNL290W</t>
+          <t>YKL056C</t>
         </is>
       </c>
     </row>
@@ -2121,7 +2121,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>YDR358W</t>
+          <t>YKR097W</t>
         </is>
       </c>
     </row>
@@ -2131,7 +2131,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>YGR239C</t>
+          <t>YDR022C</t>
         </is>
       </c>
     </row>
@@ -2141,7 +2141,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>YGR009C</t>
+          <t>YCR033W</t>
         </is>
       </c>
     </row>
@@ -2151,7 +2151,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>YHR160C</t>
+          <t>YBR214W</t>
         </is>
       </c>
     </row>
@@ -2161,7 +2161,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>YHR090C</t>
+          <t>YER020W</t>
         </is>
       </c>
     </row>
@@ -2171,7 +2171,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>YJR104C</t>
+          <t>YDR380W</t>
         </is>
       </c>
     </row>
@@ -2181,7 +2181,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>YLL018C-A</t>
+          <t>YDR098C</t>
         </is>
       </c>
     </row>
@@ -2191,7 +2191,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>YDL087C</t>
+          <t>YJL145W</t>
         </is>
       </c>
     </row>
@@ -2201,7 +2201,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>YOR076C</t>
+          <t>YOR119C</t>
         </is>
       </c>
     </row>
@@ -2211,7 +2211,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>YGR019W</t>
+          <t>YNL207W</t>
         </is>
       </c>
     </row>
@@ -2221,7 +2221,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>YJL005W</t>
+          <t>YOL055C</t>
         </is>
       </c>
     </row>
@@ -2231,7 +2231,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>YKR021W</t>
+          <t>YLR330W</t>
         </is>
       </c>
     </row>
@@ -2241,7 +2241,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>YJR032W</t>
+          <t>YNL074C</t>
         </is>
       </c>
     </row>
@@ -2251,7 +2251,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>YBR151W</t>
+          <t>YLL010C</t>
         </is>
       </c>
     </row>
@@ -2261,7 +2261,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>YDR196C</t>
+          <t>YGL045W</t>
         </is>
       </c>
     </row>
@@ -2271,7 +2271,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>YGL258W</t>
+          <t>YBR272C</t>
         </is>
       </c>
     </row>
@@ -2281,7 +2281,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>YLR027C</t>
+          <t>YDL226C</t>
         </is>
       </c>
     </row>
@@ -2291,7 +2291,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>YKR026C</t>
+          <t>YGR074W</t>
         </is>
       </c>
     </row>
@@ -2301,7 +2301,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>YCL034W</t>
+          <t>YGL015C</t>
         </is>
       </c>
     </row>
@@ -2311,7 +2311,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>YDR380W</t>
+          <t>YNL015W</t>
         </is>
       </c>
     </row>
@@ -2321,7 +2321,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>YNR070W</t>
+          <t>YNL258C</t>
         </is>
       </c>
     </row>
@@ -2331,7 +2331,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>YHR133C</t>
+          <t>YLL001W</t>
         </is>
       </c>
     </row>
@@ -2341,7 +2341,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>YGR083C</t>
+          <t>YIL143C</t>
         </is>
       </c>
     </row>
@@ -2351,7 +2351,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>YGR274C</t>
+          <t>YAL035W</t>
         </is>
       </c>
     </row>
@@ -2361,7 +2361,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>YGR261C</t>
+          <t>YJL102W</t>
         </is>
       </c>
     </row>
@@ -2371,7 +2371,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>YKL062W</t>
+          <t>YOR115C</t>
         </is>
       </c>
     </row>
@@ -2381,7 +2381,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>YJR006W</t>
+          <t>YPL111W</t>
         </is>
       </c>
     </row>
@@ -2391,7 +2391,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>YNL282W</t>
+          <t>YMR304W</t>
         </is>
       </c>
     </row>
@@ -2401,7 +2401,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>YBR149W</t>
+          <t>YFL049W</t>
         </is>
       </c>
     </row>
@@ -2411,7 +2411,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>YLL036C</t>
+          <t>YCL040W</t>
         </is>
       </c>
     </row>
@@ -2421,7 +2421,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>YER020W</t>
+          <t>YBR172C</t>
         </is>
       </c>
     </row>
@@ -2431,7 +2431,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>YHL043W</t>
+          <t>YNL035C</t>
         </is>
       </c>
     </row>
@@ -2441,7 +2441,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>YNL207W</t>
+          <t>YPL065W</t>
         </is>
       </c>
     </row>
@@ -2451,7 +2451,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>YJR009C</t>
+          <t>YDR372C</t>
         </is>
       </c>
     </row>
@@ -2461,7 +2461,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>YFR022W</t>
+          <t>YHR016C</t>
         </is>
       </c>
     </row>
@@ -2471,7 +2471,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>YGL015C</t>
+          <t>YIL104C</t>
         </is>
       </c>
     </row>
@@ -2481,7 +2481,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>YDR180W</t>
+          <t>YPL100W</t>
         </is>
       </c>
     </row>
@@ -2491,7 +2491,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>YIL041W</t>
+          <t>YIL007C</t>
         </is>
       </c>
     </row>
@@ -2501,7 +2501,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>YDL022W</t>
+          <t>YOL115W</t>
         </is>
       </c>
     </row>
@@ -2511,7 +2511,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>YDR211W</t>
+          <t>YJL029C</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>YMR182C</t>
+          <t>YDR422C</t>
         </is>
       </c>
     </row>
@@ -2531,7 +2531,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>YMR208W</t>
+          <t>YDR228C</t>
         </is>
       </c>
     </row>
@@ -2541,7 +2541,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>YKL182W</t>
+          <t>YHR170W</t>
         </is>
       </c>
     </row>
@@ -2551,7 +2551,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>YLR330W</t>
+          <t>YGR093W</t>
         </is>
       </c>
     </row>
@@ -2561,7 +2561,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>YPR030W</t>
+          <t>YDL009C</t>
         </is>
       </c>
     </row>
@@ -2571,7 +2571,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>YIL026C</t>
+          <t>YGR134W</t>
         </is>
       </c>
     </row>
@@ -2581,7 +2581,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>YGL099W</t>
+          <t>YLL036C</t>
         </is>
       </c>
     </row>
@@ -2591,7 +2591,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>YNL293W</t>
+          <t>YBR105C</t>
         </is>
       </c>
     </row>
@@ -2601,7 +2601,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>YNL247W</t>
+          <t>YDL005C</t>
         </is>
       </c>
     </row>
@@ -2611,7 +2611,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>YGL045W</t>
+          <t>YPR185W</t>
         </is>
       </c>
     </row>
@@ -2621,7 +2621,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>YHR155W</t>
+          <t>YNL231C</t>
         </is>
       </c>
     </row>
@@ -2631,7 +2631,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>YAL005C</t>
+          <t>YBL078C</t>
         </is>
       </c>
     </row>
@@ -2641,7 +2641,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>YGR248W</t>
+          <t>YDR073W</t>
         </is>
       </c>
     </row>
@@ -2651,7 +2651,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>YER040W</t>
+          <t>YHR133C</t>
         </is>
       </c>
     </row>
@@ -2661,7 +2661,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>YPL091W</t>
+          <t>YPR176C</t>
         </is>
       </c>
     </row>
@@ -2671,7 +2671,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>YLL024C</t>
+          <t>YJL121C</t>
         </is>
       </c>
     </row>
@@ -2681,7 +2681,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>YDR472W</t>
+          <t>YDL065C</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>YDR195W</t>
+          <t>YKL176C</t>
         </is>
       </c>
     </row>
@@ -2701,7 +2701,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>YDR295C</t>
+          <t>YDR452W</t>
         </is>
       </c>
     </row>
@@ -2711,7 +2711,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>YCL008C</t>
+          <t>YHR030C</t>
         </is>
       </c>
     </row>
@@ -2721,7 +2721,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>YNL117W</t>
+          <t>YDR427W</t>
         </is>
       </c>
     </row>
@@ -2731,7 +2731,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>YDR484W</t>
+          <t>YDR079C-A</t>
         </is>
       </c>
     </row>
@@ -2741,7 +2741,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>YML102W</t>
+          <t>YGR009C</t>
         </is>
       </c>
     </row>
@@ -2751,7 +2751,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>YLR131C</t>
+          <t>YGR048W</t>
         </is>
       </c>
     </row>
@@ -2761,7 +2761,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>YHR035W</t>
+          <t>YLR301W</t>
         </is>
       </c>
     </row>
@@ -2771,7 +2771,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>YDR141C</t>
+          <t>YLR131C</t>
         </is>
       </c>
     </row>
@@ -2781,7 +2781,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>YKL067W</t>
+          <t>YER040W</t>
         </is>
       </c>
     </row>
@@ -2791,7 +2791,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>YNL167C</t>
+          <t>YDR373W</t>
         </is>
       </c>
     </row>
@@ -2801,7 +2801,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>YAR007C</t>
+          <t>YHR018C</t>
         </is>
       </c>
     </row>
@@ -2811,7 +2811,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>YGL008C</t>
+          <t>YGR144W</t>
         </is>
       </c>
     </row>
@@ -2821,7 +2821,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>YNL264C</t>
+          <t>YBR056W</t>
         </is>
       </c>
     </row>
@@ -2831,7 +2831,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>YNR010W</t>
+          <t>YGR057C</t>
         </is>
       </c>
     </row>
@@ -2841,7 +2841,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>YDR267C</t>
+          <t>YNL300W</t>
         </is>
       </c>
     </row>
@@ -2851,7 +2851,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>YGR037C</t>
+          <t>YOR394W</t>
         </is>
       </c>
     </row>
@@ -2861,7 +2861,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>YNL258C</t>
+          <t>YGL246C</t>
         </is>
       </c>
     </row>
@@ -2871,7 +2871,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>YPL138C</t>
+          <t>YNL183C</t>
         </is>
       </c>
     </row>
@@ -2881,7 +2881,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>YBL091C-A</t>
+          <t>YLR153C</t>
         </is>
       </c>
     </row>
@@ -2891,7 +2891,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>YDR073W</t>
+          <t>YBR289W</t>
         </is>
       </c>
     </row>
@@ -2901,7 +2901,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>YPL262W</t>
+          <t>YEL018W</t>
         </is>
       </c>
     </row>
@@ -2911,7 +2911,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>YER025W</t>
+          <t>YLR376C</t>
         </is>
       </c>
     </row>
@@ -2921,7 +2921,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>YOR094W</t>
+          <t>YEL021W</t>
         </is>
       </c>
     </row>
@@ -2931,7 +2931,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>YMR023C</t>
+          <t>YBR151W</t>
         </is>
       </c>
     </row>
@@ -2941,7 +2941,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>YMR120C</t>
+          <t>YIR007W</t>
         </is>
       </c>
     </row>
@@ -2951,7 +2951,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>YNL300W</t>
+          <t>YEL046C</t>
         </is>
       </c>
     </row>
@@ -2961,7 +2961,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>YKL059C</t>
+          <t>YAR007C</t>
         </is>
       </c>
     </row>
@@ -2971,7 +2971,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>YPR180W</t>
+          <t>YJL031C</t>
         </is>
       </c>
     </row>
@@ -2981,7 +2981,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>YJL088W</t>
+          <t>YDR255C</t>
         </is>
       </c>
     </row>
@@ -2991,7 +2991,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>YMR029C</t>
+          <t>YPL138C</t>
         </is>
       </c>
     </row>
@@ -3001,7 +3001,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>YLR262C</t>
+          <t>YLR151C</t>
         </is>
       </c>
     </row>
@@ -3011,7 +3011,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>YPR080W</t>
+          <t>YHR035W</t>
         </is>
       </c>
     </row>
@@ -3021,7 +3021,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>YHR016C</t>
+          <t>YGL220W</t>
         </is>
       </c>
     </row>
@@ -3031,7 +3031,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>YGR254W</t>
+          <t>YDR069C</t>
         </is>
       </c>
     </row>
@@ -3041,7 +3041,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>YNL227C</t>
+          <t>YDL108W</t>
         </is>
       </c>
     </row>
@@ -3051,7 +3051,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>YOR157C</t>
+          <t>YNL216W</t>
         </is>
       </c>
     </row>
@@ -3061,7 +3061,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>YCL055W</t>
+          <t>YMR016C</t>
         </is>
       </c>
     </row>
@@ -3071,7 +3071,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>YCL011C</t>
+          <t>YDL106C</t>
         </is>
       </c>
     </row>
@@ -3081,7 +3081,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>YDR218C</t>
+          <t>YDL022C-A</t>
         </is>
       </c>
     </row>
@@ -3091,7 +3091,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>YPL175W</t>
+          <t>YDL234C</t>
         </is>
       </c>
     </row>
@@ -3101,7 +3101,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>YDL022C-A</t>
+          <t>YGL112C</t>
         </is>
       </c>
     </row>
@@ -3111,7 +3111,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>YLR019W</t>
+          <t>YPL091W</t>
         </is>
       </c>
     </row>
@@ -3121,7 +3121,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>YGR142W</t>
+          <t>YBR236C</t>
         </is>
       </c>
     </row>
@@ -3131,7 +3131,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>YGR252W</t>
+          <t>YPR080W</t>
         </is>
       </c>
     </row>
@@ -3141,7 +3141,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>YKL126W</t>
+          <t>YNR035C</t>
         </is>
       </c>
     </row>
@@ -3151,7 +3151,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>YBL078C</t>
+          <t>YOR388C</t>
         </is>
       </c>
     </row>
@@ -3161,7 +3161,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>YEL022W</t>
+          <t>YJL011C</t>
         </is>
       </c>
     </row>
@@ -3171,7 +3171,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>YLL010C</t>
+          <t>YKL022C</t>
         </is>
       </c>
     </row>
@@ -3181,7 +3181,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>YGR209C</t>
+          <t>YNL329C</t>
         </is>
       </c>
     </row>
@@ -3191,7 +3191,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>YMR173W</t>
+          <t>YHL043W</t>
         </is>
       </c>
     </row>
@@ -3201,7 +3201,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>YIL063C</t>
+          <t>YMR018W</t>
         </is>
       </c>
     </row>
@@ -3211,7 +3211,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>YLR174W</t>
+          <t>YBL001C</t>
         </is>
       </c>
     </row>
@@ -3221,7 +3221,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>YDR490C</t>
+          <t>YOR076C</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>YPL070W</t>
+          <t>YNL293W</t>
         </is>
       </c>
     </row>
@@ -3241,7 +3241,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>YEL013W</t>
+          <t>YKR068C</t>
         </is>
       </c>
     </row>
@@ -3251,7 +3251,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>YDL135C</t>
+          <t>YJL205C</t>
         </is>
       </c>
     </row>
@@ -3261,7 +3261,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>YDL100C</t>
+          <t>YGL047W</t>
         </is>
       </c>
     </row>
@@ -3271,7 +3271,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>YKR020W</t>
+          <t>YPL088W</t>
         </is>
       </c>
     </row>
@@ -3281,7 +3281,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>YGR144W</t>
+          <t>YPL153C</t>
         </is>
       </c>
     </row>
@@ -3291,7 +3291,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>YPL123C</t>
+          <t>YPL203W</t>
         </is>
       </c>
     </row>
@@ -3301,7 +3301,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>YIL036W</t>
+          <t>YOR357C</t>
         </is>
       </c>
     </row>
@@ -3311,7 +3311,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>YJR072C</t>
+          <t>YML071C</t>
         </is>
       </c>
     </row>
@@ -3321,7 +3321,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>YNL273W</t>
+          <t>YBL058W</t>
         </is>
       </c>
     </row>
@@ -3331,7 +3331,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>YDR513W</t>
+          <t>YGR261C</t>
         </is>
       </c>
     </row>
@@ -3341,7 +3341,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>YPR107C</t>
+          <t>YCR073W-A</t>
         </is>
       </c>
     </row>
@@ -3351,7 +3351,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>YBR289W</t>
+          <t>YLL009C</t>
         </is>
       </c>
     </row>
@@ -3361,7 +3361,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>YGL180W</t>
+          <t>YNL068C</t>
         </is>
       </c>
     </row>
@@ -3371,7 +3371,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>YKR080W</t>
+          <t>YPR030W</t>
         </is>
       </c>
     </row>
@@ -3381,7 +3381,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>YNL183C</t>
+          <t>YJR141W</t>
         </is>
       </c>
     </row>
@@ -3391,7 +3391,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>YGR134W</t>
+          <t>YGR198W</t>
         </is>
       </c>
     </row>
@@ -3401,7 +3401,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>YIR004W</t>
+          <t>YJL159W</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>YFR053C</t>
+          <t>YKL041W</t>
         </is>
       </c>
     </row>
@@ -3421,7 +3421,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>YML028W</t>
+          <t>YOR274W</t>
         </is>
       </c>
     </row>
@@ -3431,7 +3431,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>YPL051W</t>
+          <t>YCL055W</t>
         </is>
       </c>
     </row>
@@ -3441,7 +3441,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>YJL038C</t>
+          <t>YDR487C</t>
         </is>
       </c>
     </row>
@@ -3451,7 +3451,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>YFR021W</t>
+          <t>YGR156W</t>
         </is>
       </c>
     </row>
@@ -3461,7 +3461,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>YOL081W</t>
+          <t>YBR080C</t>
         </is>
       </c>
     </row>
@@ -3471,7 +3471,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>YDR096W</t>
+          <t>YNL167C</t>
         </is>
       </c>
     </row>
@@ -3481,7 +3481,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>YJL061W</t>
+          <t>YLR396C</t>
         </is>
       </c>
     </row>
@@ -3491,7 +3491,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>YJL121C</t>
+          <t>YMR076C</t>
         </is>
       </c>
     </row>
@@ -3501,7 +3501,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>YDR228C</t>
+          <t>YLR027C</t>
         </is>
       </c>
     </row>
@@ -3511,7 +3511,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>YBR261C</t>
+          <t>YDR484W</t>
         </is>
       </c>
     </row>
@@ -3521,7 +3521,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>YDL005C</t>
+          <t>YHR055C</t>
         </is>
       </c>
     </row>
@@ -3531,7 +3531,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>YOL115W</t>
+          <t>YCL018W</t>
         </is>
       </c>
     </row>
@@ -3541,7 +3541,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>YLR309C</t>
+          <t>YOL082W</t>
         </is>
       </c>
     </row>
@@ -3551,7 +3551,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>YNR007C</t>
+          <t>YNL051W</t>
         </is>
       </c>
     </row>
@@ -3561,7 +3561,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>YGL211W</t>
+          <t>YHR197W</t>
         </is>
       </c>
     </row>
@@ -3571,7 +3571,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>YCR043C</t>
+          <t>YML131W</t>
         </is>
       </c>
     </row>
@@ -3581,7 +3581,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>YOR274W</t>
+          <t>YIL118W</t>
         </is>
       </c>
     </row>
@@ -3591,7 +3591,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>YHR005C</t>
+          <t>YHR001W</t>
         </is>
       </c>
     </row>
@@ -3601,7 +3601,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>YDR216W</t>
+          <t>YLR039C</t>
         </is>
       </c>
     </row>
@@ -3611,7 +3611,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>YGR058W</t>
+          <t>YKR026C</t>
         </is>
       </c>
     </row>
@@ -3621,7 +3621,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>YGL124C</t>
+          <t>YMR068W</t>
         </is>
       </c>
     </row>
@@ -3631,7 +3631,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>YKL197C</t>
+          <t>YLR438W</t>
         </is>
       </c>
     </row>
@@ -3641,7 +3641,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>YOR359W</t>
+          <t>YPR103W</t>
         </is>
       </c>
     </row>
@@ -3651,7 +3651,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>YDR403W</t>
+          <t>YPL262W</t>
         </is>
       </c>
     </row>
@@ -3661,7 +3661,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>YGL253W</t>
+          <t>YKL196C</t>
         </is>
       </c>
     </row>
@@ -3671,7 +3671,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>YMR018W</t>
+          <t>YDR244W</t>
         </is>
       </c>
     </row>
@@ -3681,7 +3681,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>YPL088W</t>
+          <t>YNR010W</t>
         </is>
       </c>
     </row>
@@ -3691,7 +3691,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>YKL069W</t>
+          <t>YMR061W</t>
         </is>
       </c>
     </row>
@@ -3701,7 +3701,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>YKR097W</t>
+          <t>YDR174W</t>
         </is>
       </c>
     </row>
@@ -3711,7 +3711,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>YGR093W</t>
+          <t>YGL258W</t>
         </is>
       </c>
     </row>
@@ -3721,7 +3721,7 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>YBR164C</t>
+          <t>YER093C</t>
         </is>
       </c>
     </row>
@@ -3731,7 +3731,7 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>YER057C</t>
+          <t>YOR113W</t>
         </is>
       </c>
     </row>
@@ -3741,7 +3741,7 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>YDR022C</t>
+          <t>YCL002C</t>
         </is>
       </c>
     </row>
@@ -3761,7 +3761,7 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>YGL108C</t>
+          <t>YNL227C</t>
         </is>
       </c>
     </row>
@@ -3771,7 +3771,7 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>YGR057C</t>
+          <t>YLR309C</t>
         </is>
       </c>
     </row>
@@ -3781,7 +3781,7 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>YKR007W</t>
+          <t>YPL061W</t>
         </is>
       </c>
     </row>
@@ -3791,7 +3791,7 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>YOR370C</t>
+          <t>YOR038C</t>
         </is>
       </c>
     </row>
@@ -3801,7 +3801,7 @@
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>YPL061W</t>
+          <t>YKL060C</t>
         </is>
       </c>
     </row>
@@ -3811,7 +3811,7 @@
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>YDR372C</t>
+          <t>YPL201C</t>
         </is>
       </c>
     </row>
@@ -3821,7 +3821,7 @@
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>YLR377C</t>
+          <t>YCL034W</t>
         </is>
       </c>
     </row>
@@ -3831,7 +3831,7 @@
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>YNL259C</t>
+          <t>YFL045C</t>
         </is>
       </c>
     </row>
@@ -3841,7 +3841,7 @@
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>YHR018C</t>
+          <t>YPL051W</t>
         </is>
       </c>
     </row>
@@ -3851,7 +3851,7 @@
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>YOR394W</t>
+          <t>YBR030W</t>
         </is>
       </c>
     </row>
@@ -3861,7 +3861,7 @@
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>YBR172C</t>
+          <t>YGR037C</t>
         </is>
       </c>
     </row>
@@ -3871,7 +3871,7 @@
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>YHR170W</t>
+          <t>YBR152W</t>
         </is>
       </c>
     </row>
@@ -3881,7 +3881,7 @@
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>YDL137W</t>
+          <t>YNR024W</t>
         </is>
       </c>
     </row>
@@ -3891,7 +3891,7 @@
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>YGR074W</t>
+          <t>YHR202W</t>
         </is>
       </c>
     </row>
@@ -3901,7 +3901,7 @@
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>YBL050W</t>
+          <t>YAL054C</t>
         </is>
       </c>
     </row>
@@ -3911,7 +3911,7 @@
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>YGR156W</t>
+          <t>YKL069W</t>
         </is>
       </c>
     </row>
@@ -3921,7 +3921,7 @@
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>YGR270W</t>
+          <t>YDR403W</t>
         </is>
       </c>
     </row>
@@ -3931,7 +3931,7 @@
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>YIR007W</t>
+          <t>YGR058W</t>
         </is>
       </c>
     </row>
@@ -3941,7 +3941,7 @@
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>YER175C</t>
+          <t>YDR295C</t>
         </is>
       </c>
     </row>
@@ -3951,7 +3951,7 @@
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>YNR049C</t>
+          <t>YHR073W</t>
         </is>
       </c>
     </row>
@@ -3961,7 +3961,7 @@
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>YEL046C</t>
+          <t>YGL095C</t>
         </is>
       </c>
     </row>
@@ -3971,7 +3971,7 @@
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>YPL065W</t>
+          <t>YKL067W</t>
         </is>
       </c>
     </row>
@@ -3981,7 +3981,7 @@
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>YHR109W</t>
+          <t>YPL249C</t>
         </is>
       </c>
     </row>
@@ -3991,7 +3991,7 @@
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>YAL035W</t>
+          <t>YHR053C</t>
         </is>
       </c>
     </row>
@@ -4001,7 +4001,7 @@
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>YOR357C</t>
+          <t>YDR142C</t>
         </is>
       </c>
     </row>
@@ -4011,7 +4011,7 @@
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>YNR034W-A</t>
+          <t>YPL117C</t>
         </is>
       </c>
     </row>
@@ -4021,7 +4021,7 @@
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>YBR105C</t>
+          <t>YIL044C</t>
         </is>
       </c>
     </row>
@@ -4031,7 +4031,7 @@
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>YKR082W</t>
+          <t>YDR517W</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>YPL140C</t>
+          <t>YGL124C</t>
         </is>
       </c>
     </row>
@@ -4051,7 +4051,7 @@
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>YHR131C</t>
+          <t>YOR069W</t>
         </is>
       </c>
     </row>
@@ -4061,7 +4061,7 @@
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>YFL049W</t>
+          <t>YOR322C</t>
         </is>
       </c>
     </row>
@@ -4071,7 +4071,7 @@
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>YFL068W</t>
+          <t>YKL026C</t>
         </is>
       </c>
     </row>
@@ -4081,7 +4081,7 @@
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>YDR373W</t>
+          <t>YIR004W</t>
         </is>
       </c>
     </row>
@@ -4091,7 +4091,7 @@
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>YNL242W</t>
+          <t>YJL061W</t>
         </is>
       </c>
     </row>
@@ -4101,7 +4101,7 @@
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>YNL246W</t>
+          <t>YDR189W</t>
         </is>
       </c>
     </row>
@@ -4111,7 +4111,7 @@
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>YMR016C</t>
+          <t>YHR160C</t>
         </is>
       </c>
     </row>
@@ -4121,7 +4121,7 @@
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>YLR116W</t>
+          <t>YMR208W</t>
         </is>
       </c>
     </row>
@@ -4131,7 +4131,7 @@
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>YJL084C</t>
+          <t>YGR241C</t>
         </is>
       </c>
     </row>
@@ -4141,7 +4141,7 @@
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>YDL065C</t>
+          <t>YOR370C</t>
         </is>
       </c>
     </row>
@@ -4151,7 +4151,7 @@
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>YDR108W</t>
+          <t>YBL018C</t>
         </is>
       </c>
     </row>
@@ -4161,7 +4161,7 @@
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>YER129W</t>
+          <t>YCL011C</t>
         </is>
       </c>
     </row>
@@ -4171,7 +4171,7 @@
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>YOR115C</t>
+          <t>YJL176C</t>
         </is>
       </c>
     </row>
@@ -4181,7 +4181,7 @@
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>YJL031C</t>
+          <t>YFR021W</t>
         </is>
       </c>
     </row>
@@ -4191,7 +4191,7 @@
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>YLR028C</t>
+          <t>YIL026C</t>
         </is>
       </c>
     </row>
@@ -4201,7 +4201,7 @@
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>YGR233C</t>
+          <t>YML028W</t>
         </is>
       </c>
     </row>
@@ -4211,7 +4211,7 @@
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>YKR071C</t>
+          <t>YBL101C</t>
         </is>
       </c>
     </row>
@@ -4221,7 +4221,7 @@
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t>YKL022C</t>
+          <t>YPL070W</t>
         </is>
       </c>
     </row>
@@ -4231,7 +4231,7 @@
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>YHR053C</t>
+          <t>YLL029W</t>
         </is>
       </c>
     </row>
@@ -4241,7 +4241,7 @@
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t>YJL052W</t>
+          <t>YPL123C</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t>YLR304C</t>
+          <t>YKR082W</t>
         </is>
       </c>
     </row>
@@ -4261,7 +4261,7 @@
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>YOR069W</t>
+          <t>YNL242W</t>
         </is>
       </c>
     </row>
@@ -4271,7 +4271,7 @@
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t>YKL176C</t>
+          <t>YPL084W</t>
         </is>
       </c>
     </row>
@@ -4281,7 +4281,7 @@
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t>YCL040W</t>
+          <t>YKL130C</t>
         </is>
       </c>
     </row>
@@ -4291,7 +4291,7 @@
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>YFL014W</t>
+          <t>YER007C-A</t>
         </is>
       </c>
     </row>
@@ -4301,7 +4301,7 @@
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>YMR235C</t>
+          <t>YMR120C</t>
         </is>
       </c>
     </row>
@@ -4311,7 +4311,7 @@
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>YDL108W</t>
+          <t>YMR023C</t>
         </is>
       </c>
     </row>
@@ -4321,7 +4321,7 @@
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>YGL083W</t>
+          <t>YPR144C</t>
         </is>
       </c>
     </row>
@@ -4331,7 +4331,7 @@
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t>YGL095C</t>
+          <t>YJL038C</t>
         </is>
       </c>
     </row>
@@ -4341,7 +4341,7 @@
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t>YJL115W</t>
+          <t>YDR195W</t>
         </is>
       </c>
     </row>
@@ -4351,7 +4351,7 @@
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t>YOL126C</t>
+          <t>YOR260W</t>
         </is>
       </c>
     </row>
@@ -4361,7 +4361,7 @@
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t>YBR017C</t>
+          <t>YGL099W</t>
         </is>
       </c>
     </row>
@@ -4371,7 +4371,7 @@
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t>YLR301W</t>
+          <t>YNL264C</t>
         </is>
       </c>
     </row>
@@ -4381,7 +4381,7 @@
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t>YNL006W</t>
+          <t>YOR168W</t>
         </is>
       </c>
     </row>
@@ -4391,7 +4391,7 @@
       </c>
       <c r="B397" t="inlineStr">
         <is>
-          <t>YPR032W</t>
+          <t>YJL044C</t>
         </is>
       </c>
     </row>
@@ -4401,7 +4401,7 @@
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t>YDL126C</t>
+          <t>YFL014W</t>
         </is>
       </c>
     </row>
@@ -4411,7 +4411,7 @@
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t>YJL029C</t>
+          <t>YDR490C</t>
         </is>
       </c>
     </row>
@@ -4421,7 +4421,7 @@
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t>YGL062W</t>
+          <t>YPR105C</t>
         </is>
       </c>
     </row>
@@ -4431,7 +4431,7 @@
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t>YIL009C-A</t>
+          <t>YNR051C</t>
         </is>
       </c>
     </row>
@@ -4441,7 +4441,7 @@
       </c>
       <c r="B402" t="inlineStr">
         <is>
-          <t>YFL045C</t>
+          <t>YLR195C</t>
         </is>
       </c>
     </row>
@@ -4451,7 +4451,7 @@
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t>YNR051C</t>
+          <t>YOL059W</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t>YDR244W</t>
+          <t>YOR122C</t>
         </is>
       </c>
     </row>
@@ -4471,7 +4471,7 @@
       </c>
       <c r="B405" t="inlineStr">
         <is>
-          <t>YLR293C</t>
+          <t>YDR196C</t>
         </is>
       </c>
     </row>
@@ -4481,7 +4481,7 @@
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t>YNL064C</t>
+          <t>YDR172W</t>
         </is>
       </c>
     </row>
@@ -4491,7 +4491,7 @@
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t>YMR038C</t>
+          <t>YLR377C</t>
         </is>
       </c>
     </row>
@@ -4501,7 +4501,7 @@
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>YDR177W</t>
+          <t>YLL024C</t>
         </is>
       </c>
     </row>
@@ -4511,7 +4511,7 @@
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>YCR073W-A</t>
+          <t>YKR007W</t>
         </is>
       </c>
     </row>
@@ -4521,7 +4521,7 @@
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>YMR068W</t>
+          <t>YKR071C</t>
         </is>
       </c>
     </row>
@@ -4531,7 +4531,7 @@
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>YDR049W</t>
+          <t>YIL084C</t>
         </is>
       </c>
     </row>
@@ -4541,7 +4541,7 @@
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t>YIL084C</t>
+          <t>YGL013C</t>
         </is>
       </c>
     </row>
@@ -4551,7 +4551,7 @@
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>YER023W</t>
+          <t>YMR043W</t>
         </is>
       </c>
     </row>
@@ -4561,7 +4561,7 @@
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>YDR098C</t>
+          <t>YER129W</t>
         </is>
       </c>
     </row>
@@ -4571,7 +4571,7 @@
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t>YKL075C</t>
+          <t>YHR150W</t>
         </is>
       </c>
     </row>
@@ -4581,7 +4581,7 @@
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t>YMR028W</t>
+          <t>YGL115W</t>
         </is>
       </c>
     </row>
@@ -4591,7 +4591,7 @@
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>YOR122C</t>
+          <t>YNL259C</t>
         </is>
       </c>
     </row>
@@ -4601,7 +4601,7 @@
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t>YOL083W</t>
+          <t>YDR392W</t>
         </is>
       </c>
     </row>
@@ -4611,7 +4611,7 @@
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>YDR487C</t>
+          <t>YEL013W</t>
         </is>
       </c>
     </row>
@@ -4621,7 +4621,7 @@
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t>YBL076C</t>
+          <t>YLR262C</t>
         </is>
       </c>
     </row>
@@ -4631,7 +4631,7 @@
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>YJL068C</t>
+          <t>YBR067C</t>
         </is>
       </c>
     </row>
@@ -4641,7 +4641,7 @@
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>YKL060C</t>
+          <t>YCR043C</t>
         </is>
       </c>
     </row>
@@ -4651,7 +4651,7 @@
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>YPR159C-A</t>
+          <t>YPL120W</t>
         </is>
       </c>
     </row>
@@ -4661,7 +4661,7 @@
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>YPL111W</t>
+          <t>YLR455W</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>YGL009C</t>
+          <t>YGL145W</t>
         </is>
       </c>
     </row>
@@ -4681,7 +4681,7 @@
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>YGL112C</t>
+          <t>YDR472W</t>
         </is>
       </c>
     </row>
@@ -4691,7 +4691,7 @@
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>YLL029W</t>
+          <t>YOL062C</t>
         </is>
       </c>
     </row>
@@ -4701,7 +4701,7 @@
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>YHR176W</t>
+          <t>YBR218C</t>
         </is>
       </c>
     </row>
@@ -4711,7 +4711,7 @@
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t>YGL004C</t>
+          <t>YIR037W</t>
         </is>
       </c>
     </row>
@@ -4721,7 +4721,7 @@
       </c>
       <c r="B430" t="inlineStr">
         <is>
-          <t>YNL272C</t>
+          <t>YBR095C</t>
         </is>
       </c>
     </row>
@@ -4731,7 +4731,7 @@
       </c>
       <c r="B431" t="inlineStr">
         <is>
-          <t>YDR300C</t>
+          <t>YOR133W</t>
         </is>
       </c>
     </row>
@@ -4741,7 +4741,7 @@
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t>YDR392W</t>
+          <t>YNL290W</t>
         </is>
       </c>
     </row>
@@ -4751,7 +4751,7 @@
       </c>
       <c r="B433" t="inlineStr">
         <is>
-          <t>YML113W</t>
+          <t>YLR028C</t>
         </is>
       </c>
     </row>
@@ -4761,7 +4761,7 @@
       </c>
       <c r="B434" t="inlineStr">
         <is>
-          <t>YPL084W</t>
+          <t>YDR311W</t>
         </is>
       </c>
     </row>
@@ -4771,7 +4771,7 @@
       </c>
       <c r="B435" t="inlineStr">
         <is>
-          <t>YMR077C</t>
+          <t>YBR149W</t>
         </is>
       </c>
     </row>
@@ -4781,7 +4781,7 @@
       </c>
       <c r="B436" t="inlineStr">
         <is>
-          <t>YNL074C</t>
+          <t>YOL053W</t>
         </is>
       </c>
     </row>
@@ -4791,7 +4791,7 @@
       </c>
       <c r="B437" t="inlineStr">
         <is>
-          <t>YJL102W</t>
+          <t>YLR109W</t>
         </is>
       </c>
     </row>
@@ -4801,7 +4801,7 @@
       </c>
       <c r="B438" t="inlineStr">
         <is>
-          <t>YBR095C</t>
+          <t>YDR180W</t>
         </is>
       </c>
     </row>
@@ -4811,7 +4811,7 @@
       </c>
       <c r="B439" t="inlineStr">
         <is>
-          <t>YLR291C</t>
+          <t>YOL138C</t>
         </is>
       </c>
     </row>
@@ -4821,7 +4821,7 @@
       </c>
       <c r="B440" t="inlineStr">
         <is>
-          <t>YJL036W</t>
+          <t>YLR310C</t>
         </is>
       </c>
     </row>
@@ -4831,7 +4831,7 @@
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t>YPL096W</t>
+          <t>YKL135C</t>
         </is>
       </c>
     </row>
@@ -4841,7 +4841,7 @@
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t>YGR120C</t>
+          <t>YIL009C-A</t>
         </is>
       </c>
     </row>
@@ -4851,7 +4851,7 @@
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t>YDR079C-A</t>
+          <t>YMR277W</t>
         </is>
       </c>
     </row>
@@ -4861,7 +4861,7 @@
       </c>
       <c r="B444" t="inlineStr">
         <is>
-          <t>YNR035C</t>
+          <t>YNL127W</t>
         </is>
       </c>
     </row>
@@ -4871,7 +4871,7 @@
       </c>
       <c r="B445" t="inlineStr">
         <is>
-          <t>YPR103W</t>
+          <t>YOR359W</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="B446" t="inlineStr">
         <is>
-          <t>YIL104C</t>
+          <t>YOR229W</t>
         </is>
       </c>
     </row>
@@ -4891,7 +4891,7 @@
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t>YMR277W</t>
+          <t>YNL282W</t>
         </is>
       </c>
     </row>
@@ -4901,7 +4901,7 @@
       </c>
       <c r="B448" t="inlineStr">
         <is>
-          <t>YHR197W</t>
+          <t>YJL005W</t>
         </is>
       </c>
     </row>
@@ -4911,7 +4911,7 @@
       </c>
       <c r="B449" t="inlineStr">
         <is>
-          <t>YDR464W</t>
+          <t>YNL006W</t>
         </is>
       </c>
     </row>
@@ -4921,7 +4921,7 @@
       </c>
       <c r="B450" t="inlineStr">
         <is>
-          <t>YHR206W</t>
+          <t>YBR261C</t>
         </is>
       </c>
     </row>
@@ -4931,7 +4931,7 @@
       </c>
       <c r="B451" t="inlineStr">
         <is>
-          <t>YDR353W</t>
+          <t>YMR037C</t>
         </is>
       </c>
     </row>
@@ -4941,7 +4941,7 @@
       </c>
       <c r="B452" t="inlineStr">
         <is>
-          <t>YBL075C</t>
+          <t>YGR129W</t>
         </is>
       </c>
     </row>
@@ -4951,7 +4951,7 @@
       </c>
       <c r="B453" t="inlineStr">
         <is>
-          <t>YGL246C</t>
+          <t>YKL113C</t>
         </is>
       </c>
     </row>
@@ -4961,7 +4961,7 @@
       </c>
       <c r="B454" t="inlineStr">
         <is>
-          <t>YLR396C</t>
+          <t>YDR165W</t>
         </is>
       </c>
     </row>
@@ -4971,7 +4971,7 @@
       </c>
       <c r="B455" t="inlineStr">
         <is>
-          <t>YFL030W</t>
+          <t>YMR235C</t>
         </is>
       </c>
     </row>
@@ -4981,7 +4981,7 @@
       </c>
       <c r="B456" t="inlineStr">
         <is>
-          <t>YLL052C</t>
+          <t>YOL083W</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4991,7 @@
       </c>
       <c r="B457" t="inlineStr">
         <is>
-          <t>YAL054C</t>
+          <t>YOL094C</t>
         </is>
       </c>
     </row>
@@ -5001,7 +5001,7 @@
       </c>
       <c r="B458" t="inlineStr">
         <is>
-          <t>YNR016C</t>
+          <t>YLR304C</t>
         </is>
       </c>
     </row>
@@ -5011,7 +5011,7 @@
       </c>
       <c r="B459" t="inlineStr">
         <is>
-          <t>YHR171W</t>
+          <t>YOR094W</t>
         </is>
       </c>
     </row>
@@ -5021,7 +5021,7 @@
       </c>
       <c r="B460" t="inlineStr">
         <is>
-          <t>YDR452W</t>
+          <t>YNL273W</t>
         </is>
       </c>
     </row>
@@ -5031,7 +5031,7 @@
       </c>
       <c r="B461" t="inlineStr">
         <is>
-          <t>YMR043W</t>
+          <t>YPL096W</t>
         </is>
       </c>
     </row>
@@ -5041,7 +5041,7 @@
       </c>
       <c r="B462" t="inlineStr">
         <is>
-          <t>YBR131W</t>
+          <t>YIR031C</t>
         </is>
       </c>
     </row>
@@ -5051,7 +5051,7 @@
       </c>
       <c r="B463" t="inlineStr">
         <is>
-          <t>YHR001W</t>
+          <t>YKR084C</t>
         </is>
       </c>
     </row>
@@ -5061,7 +5061,7 @@
       </c>
       <c r="B464" t="inlineStr">
         <is>
-          <t>YCL018W</t>
+          <t>YAR002W</t>
         </is>
       </c>
     </row>
@@ -5071,7 +5071,7 @@
       </c>
       <c r="B465" t="inlineStr">
         <is>
-          <t>YER007C-A</t>
+          <t>YDR320C</t>
         </is>
       </c>
     </row>
@@ -5081,7 +5081,7 @@
       </c>
       <c r="B466" t="inlineStr">
         <is>
-          <t>YJR102C</t>
+          <t>YFL013C</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="B467" t="inlineStr">
         <is>
-          <t>YOR260W</t>
+          <t>YJL052W</t>
         </is>
       </c>
     </row>
@@ -5101,7 +5101,7 @@
       </c>
       <c r="B468" t="inlineStr">
         <is>
-          <t>YKL041W</t>
+          <t>YEL047C</t>
         </is>
       </c>
     </row>
@@ -5111,7 +5111,7 @@
       </c>
       <c r="B469" t="inlineStr">
         <is>
-          <t>YJL208C</t>
+          <t>YJL036W</t>
         </is>
       </c>
     </row>
@@ -5121,7 +5121,7 @@
       </c>
       <c r="B470" t="inlineStr">
         <is>
-          <t>YPL203W</t>
+          <t>YLR240W</t>
         </is>
       </c>
     </row>
@@ -5131,7 +5131,7 @@
       </c>
       <c r="B471" t="inlineStr">
         <is>
-          <t>YBR152W</t>
+          <t>YBR164C</t>
         </is>
       </c>
     </row>
@@ -5141,7 +5141,7 @@
       </c>
       <c r="B472" t="inlineStr">
         <is>
-          <t>YDR334W</t>
+          <t>YAL005C</t>
         </is>
       </c>
     </row>
@@ -5151,7 +5151,7 @@
       </c>
       <c r="B473" t="inlineStr">
         <is>
-          <t>YLL038C</t>
+          <t>YKL062W</t>
         </is>
       </c>
     </row>
@@ -5161,7 +5161,7 @@
       </c>
       <c r="B474" t="inlineStr">
         <is>
-          <t>YNR023W</t>
+          <t>YBR231C</t>
         </is>
       </c>
     </row>
@@ -5171,7 +5171,7 @@
       </c>
       <c r="B475" t="inlineStr">
         <is>
-          <t>YKR068C</t>
+          <t>YGR234W</t>
         </is>
       </c>
     </row>
@@ -5181,7 +5181,7 @@
       </c>
       <c r="B476" t="inlineStr">
         <is>
-          <t>YPL249C</t>
+          <t>YPR180W</t>
         </is>
       </c>
     </row>
@@ -5191,7 +5191,7 @@
       </c>
       <c r="B477" t="inlineStr">
         <is>
-          <t>YDR422C</t>
+          <t>YNL240C</t>
         </is>
       </c>
     </row>
@@ -5201,7 +5201,7 @@
       </c>
       <c r="B478" t="inlineStr">
         <is>
-          <t>YDL192W</t>
+          <t>YCL058C</t>
         </is>
       </c>
     </row>
@@ -5211,7 +5211,7 @@
       </c>
       <c r="B479" t="inlineStr">
         <is>
-          <t>YJR141W</t>
+          <t>YNL097C-B</t>
         </is>
       </c>
     </row>
@@ -5221,7 +5221,7 @@
       </c>
       <c r="B480" t="inlineStr">
         <is>
-          <t>YPR010C-A</t>
+          <t>YOR093C</t>
         </is>
       </c>
     </row>
@@ -5231,7 +5231,7 @@
       </c>
       <c r="B481" t="inlineStr">
         <is>
-          <t>YGR030C</t>
+          <t>YER057C</t>
         </is>
       </c>
     </row>
@@ -5241,7 +5241,7 @@
       </c>
       <c r="B482" t="inlineStr">
         <is>
-          <t>YPL231W</t>
+          <t>YER024W</t>
         </is>
       </c>
     </row>
@@ -5251,7 +5251,7 @@
       </c>
       <c r="B483" t="inlineStr">
         <is>
-          <t>YDL106C</t>
+          <t>YFL030W</t>
         </is>
       </c>
     </row>
@@ -5261,7 +5261,7 @@
       </c>
       <c r="B484" t="inlineStr">
         <is>
-          <t>YDR172W</t>
+          <t>YGL066W</t>
         </is>
       </c>
     </row>
@@ -5271,7 +5271,7 @@
       </c>
       <c r="B485" t="inlineStr">
         <is>
-          <t>YIL007C</t>
+          <t>YDR416W</t>
         </is>
       </c>
     </row>
@@ -5281,7 +5281,7 @@
       </c>
       <c r="B486" t="inlineStr">
         <is>
-          <t>YMR070W</t>
+          <t>YCR020C</t>
         </is>
       </c>
     </row>
@@ -5291,7 +5291,7 @@
       </c>
       <c r="B487" t="inlineStr">
         <is>
-          <t>YCR032W</t>
+          <t>YLR116W</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="B488" t="inlineStr">
         <is>
-          <t>YNR024W</t>
+          <t>YIR012W</t>
         </is>
       </c>
     </row>
@@ -5311,7 +5311,7 @@
       </c>
       <c r="B489" t="inlineStr">
         <is>
-          <t>YDR311W</t>
+          <t>YIL036W</t>
         </is>
       </c>
     </row>
@@ -5321,7 +5321,7 @@
       </c>
       <c r="B490" t="inlineStr">
         <is>
-          <t>YKL206C</t>
+          <t>YNL246W</t>
         </is>
       </c>
     </row>
@@ -5331,7 +5331,7 @@
       </c>
       <c r="B491" t="inlineStr">
         <is>
-          <t>YLR455W</t>
+          <t>YDR513W</t>
         </is>
       </c>
     </row>
@@ -5341,7 +5341,7 @@
       </c>
       <c r="B492" t="inlineStr">
         <is>
-          <t>YOL055C</t>
+          <t>YER023W</t>
         </is>
       </c>
     </row>
@@ -5351,7 +5351,7 @@
       </c>
       <c r="B493" t="inlineStr">
         <is>
-          <t>YAR002W</t>
+          <t>YKL075C</t>
         </is>
       </c>
     </row>
@@ -5361,7 +5361,7 @@
       </c>
       <c r="B494" t="inlineStr">
         <is>
-          <t>YMR076C</t>
+          <t>YDR464W</t>
         </is>
       </c>
     </row>
@@ -5371,7 +5371,7 @@
       </c>
       <c r="B495" t="inlineStr">
         <is>
-          <t>YLR260W</t>
+          <t>YGR209C</t>
         </is>
       </c>
     </row>
@@ -5381,7 +5381,7 @@
       </c>
       <c r="B496" t="inlineStr">
         <is>
-          <t>YPR176C</t>
+          <t>YDL087C</t>
         </is>
       </c>
     </row>
@@ -5391,7 +5391,7 @@
       </c>
       <c r="B497" t="inlineStr">
         <is>
-          <t>YDR255C</t>
+          <t>YGR059W</t>
         </is>
       </c>
     </row>
@@ -5401,7 +5401,7 @@
       </c>
       <c r="B498" t="inlineStr">
         <is>
-          <t>YBR101C</t>
+          <t>YIL041W</t>
         </is>
       </c>
     </row>
@@ -5411,7 +5411,7 @@
       </c>
       <c r="B499" t="inlineStr">
         <is>
-          <t>YOL053W</t>
+          <t>YHR206W</t>
         </is>
       </c>
     </row>
@@ -5421,7 +5421,7 @@
       </c>
       <c r="B500" t="inlineStr">
         <is>
-          <t>YER024W</t>
+          <t>YJL088W</t>
         </is>
       </c>
     </row>
@@ -5431,7 +5431,7 @@
       </c>
       <c r="B501" t="inlineStr">
         <is>
-          <t>YLR195C</t>
+          <t>YOR302W</t>
         </is>
       </c>
     </row>
@@ -5441,7 +5441,7 @@
       </c>
       <c r="B502" t="inlineStr">
         <is>
-          <t>YIL118W</t>
+          <t>YPR159C-A</t>
         </is>
       </c>
     </row>
@@ -5451,7 +5451,7 @@
       </c>
       <c r="B503" t="inlineStr">
         <is>
-          <t>YGL145W</t>
+          <t>YNR023W</t>
         </is>
       </c>
     </row>
@@ -5461,7 +5461,7 @@
       </c>
       <c r="B504" t="inlineStr">
         <is>
-          <t>YER048C</t>
+          <t>YBR017C</t>
         </is>
       </c>
     </row>
@@ -5471,7 +5471,7 @@
       </c>
       <c r="B505" t="inlineStr">
         <is>
-          <t>YML131W</t>
+          <t>YNL247W</t>
         </is>
       </c>
     </row>
@@ -5481,7 +5481,7 @@
       </c>
       <c r="B506" t="inlineStr">
         <is>
-          <t>YKL026C</t>
+          <t>YGL253W</t>
         </is>
       </c>
     </row>
@@ -5491,7 +5491,7 @@
       </c>
       <c r="B507" t="inlineStr">
         <is>
-          <t>YNL068C</t>
+          <t>YMR029C</t>
         </is>
       </c>
     </row>
@@ -5501,7 +5501,7 @@
       </c>
       <c r="B508" t="inlineStr">
         <is>
-          <t>YJL044C</t>
+          <t>YGR068C</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="B509" t="inlineStr">
         <is>
-          <t>YDR165W</t>
+          <t>YBL041W</t>
         </is>
       </c>
     </row>
@@ -5521,7 +5521,7 @@
       </c>
       <c r="B510" t="inlineStr">
         <is>
-          <t>YOL082W</t>
+          <t>YNR016C</t>
         </is>
       </c>
     </row>
@@ -5531,7 +5531,7 @@
       </c>
       <c r="B511" t="inlineStr">
         <is>
-          <t>YEL021W</t>
+          <t>YER151C</t>
         </is>
       </c>
     </row>
@@ -5541,7 +5541,7 @@
       </c>
       <c r="B512" t="inlineStr">
         <is>
-          <t>YDR174W</t>
+          <t>YMR028W</t>
         </is>
       </c>
     </row>
@@ -5551,7 +5551,7 @@
       </c>
       <c r="B513" t="inlineStr">
         <is>
-          <t>YNL015W</t>
+          <t>YDR218C</t>
         </is>
       </c>
     </row>
@@ -5561,7 +5561,7 @@
       </c>
       <c r="B514" t="inlineStr">
         <is>
-          <t>YOR038C</t>
+          <t>YKL182W</t>
         </is>
       </c>
     </row>
@@ -5571,7 +5571,7 @@
       </c>
       <c r="B515" t="inlineStr">
         <is>
-          <t>YML071C</t>
+          <t>YGR270W</t>
         </is>
       </c>
     </row>
@@ -5581,7 +5581,7 @@
       </c>
       <c r="B516" t="inlineStr">
         <is>
-          <t>YFR004W</t>
+          <t>YLR044C</t>
         </is>
       </c>
     </row>

</xml_diff>